<commit_message>
refactor(ia): auditar comercio exterior, compactar OEA y unificar termino gestion
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -775,7 +775,7 @@
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>TOTAL CONTENIDOS
-716 Trámites</t>
+715 Trámites</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -787,7 +787,7 @@
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>COMERCIO EXTERIOR
-246 Trámites</t>
+245 Trámites</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="G11" s="15" t="n">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H11" s="16">
         <f>G11/$G$15</f>
@@ -1090,7 +1090,7 @@
       <c r="E21" s="33" t="n"/>
       <c r="F21" s="33" t="n"/>
       <c r="G21" s="15" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H21" s="16">
         <f>G21/$G$24</f>
@@ -1211,7 +1211,7 @@
       <c r="E28" s="35" t="n"/>
       <c r="F28" s="35" t="n"/>
       <c r="G28" s="22" t="n">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="H28" s="23">
         <f>G28/$G$32</f>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="G19" s="15" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H19" s="38">
         <f>G19/$G$25</f>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="J38" s="48" t="inlineStr">
         <is>
-          <t>716 Trámites 100% Mapeados</t>
+          <t>715 Trámites 100% Mapeados</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
         </is>
       </c>
       <c r="H18" s="22" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" ht="54" customHeight="1">

</xml_diff>

<commit_message>
feat(ia, datos, excel): reestructurar taxonomia numerica N1-N5 y agregar fichas por nivel
- AGENTS.md: nueva regla - los niveles no llevan nombre conceptual (solo Nivel 1..Nivel 5)

- database: arbol canonico y coleccion nosql regenerados y sincronizados

- src/data: allTramites y catalogoContenidosUnicos actualizados; nuevo taxonomyDescriptions.ts

- docs: Excel del Mapa incorpora la hoja 'Fichas por Nivel' (Nivel 1-3, 40 nodos)

- scripts: generadores de taxonomia, fichas por nivel y normalizacion de ids/etiquetas

- src/pages: ajustes en PortalFlowPage y ArchitectureDiagramPage; test a11y
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen Arquitectura" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa de Navegación" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fichas por Rol y Categoría" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fichas por Nivel" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fichas por Rol y Categoría'!$A$6:$H$33</definedName>
@@ -23,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,8 +96,28 @@
       <color rgb="001E293B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -157,8 +178,38 @@
         <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0019324B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0014649B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF3FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2E8F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -252,11 +303,127 @@
         <color rgb="0064748B"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C3D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7C3D0"/>
+      </right>
+      <top style="medium">
+        <color rgb="0014649B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="0014649B"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C3D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7C3D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7C3D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7C3D0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="0014649B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B7C3D0"/>
+      </right>
+      <top style="medium">
+        <color rgb="0014649B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="0014649B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="0014649B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B7C3D0"/>
+      </right>
+      <top style="medium">
+        <color rgb="0014649B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="0014649B"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -377,6 +544,59 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1042,9 +1262,9 @@
           <t>Primer NIT, RTU Digital, padrones de importación/exportación y habilitación inicial</t>
         </is>
       </c>
-      <c r="D19" s="33" t="n"/>
-      <c r="E19" s="33" t="n"/>
-      <c r="F19" s="33" t="n"/>
+      <c r="D19" s="53" t="n"/>
+      <c r="E19" s="53" t="n"/>
+      <c r="F19" s="54" t="n"/>
       <c r="G19" s="15" t="n">
         <v>72</v>
       </c>
@@ -1064,9 +1284,9 @@
           <t>Facturación FEL, Declaraguate, DUCAs, retenciones, transferencias y pagos</t>
         </is>
       </c>
-      <c r="D20" s="35" t="n"/>
-      <c r="E20" s="35" t="n"/>
-      <c r="F20" s="35" t="n"/>
+      <c r="D20" s="53" t="n"/>
+      <c r="E20" s="53" t="n"/>
+      <c r="F20" s="54" t="n"/>
       <c r="G20" s="22" t="n">
         <v>260</v>
       </c>
@@ -1086,9 +1306,9 @@
           <t>Verificadores en tiempo real, solvencia, selectivo aduanero, rampa y SAC</t>
         </is>
       </c>
-      <c r="D21" s="33" t="n"/>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="33" t="n"/>
+      <c r="D21" s="53" t="n"/>
+      <c r="E21" s="53" t="n"/>
+      <c r="F21" s="54" t="n"/>
       <c r="G21" s="15" t="n">
         <v>116</v>
       </c>
@@ -1108,9 +1328,9 @@
           <t>Actualización de RTU, traspaso vehicular, prórrogas, cese de actividades y subastas</t>
         </is>
       </c>
-      <c r="D22" s="35" t="n"/>
-      <c r="E22" s="35" t="n"/>
-      <c r="F22" s="35" t="n"/>
+      <c r="D22" s="53" t="n"/>
+      <c r="E22" s="53" t="n"/>
+      <c r="F22" s="54" t="n"/>
       <c r="G22" s="22" t="n">
         <v>137</v>
       </c>
@@ -1130,9 +1350,9 @@
           <t>Marco legal aduanero y tributario, devoluciones, criterios institucionales y cursos</t>
         </is>
       </c>
-      <c r="D23" s="33" t="n"/>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="33" t="n"/>
+      <c r="D23" s="53" t="n"/>
+      <c r="E23" s="53" t="n"/>
+      <c r="F23" s="54" t="n"/>
       <c r="G23" s="15" t="n">
         <v>130</v>
       </c>
@@ -1152,9 +1372,9 @@
           <t>100% de contenidos clasificados según ciclo de vida</t>
         </is>
       </c>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="24" t="n"/>
-      <c r="F24" s="24" t="n"/>
+      <c r="D24" s="53" t="n"/>
+      <c r="E24" s="53" t="n"/>
+      <c r="F24" s="54" t="n"/>
       <c r="G24" s="27">
         <f>SUM(G19:G23)</f>
         <v/>
@@ -1207,9 +1427,9 @@
           <t>Páginas explicativas, requisitos de trámites presenciales o mixtos</t>
         </is>
       </c>
-      <c r="D28" s="35" t="n"/>
-      <c r="E28" s="35" t="n"/>
-      <c r="F28" s="35" t="n"/>
+      <c r="D28" s="53" t="n"/>
+      <c r="E28" s="53" t="n"/>
+      <c r="F28" s="54" t="n"/>
       <c r="G28" s="22" t="n">
         <v>490</v>
       </c>
@@ -1229,9 +1449,9 @@
           <t>Servicios digitales transaccionales (Agencia Virtual, Declaraguate, TEV, FEL)</t>
         </is>
       </c>
-      <c r="D29" s="33" t="n"/>
-      <c r="E29" s="33" t="n"/>
-      <c r="F29" s="33" t="n"/>
+      <c r="D29" s="53" t="n"/>
+      <c r="E29" s="53" t="n"/>
+      <c r="F29" s="54" t="n"/>
       <c r="G29" s="15" t="n">
         <v>137</v>
       </c>
@@ -1251,9 +1471,9 @@
           <t>Herramientas de verificación sin autenticación previa (RTU público, solvencias)</t>
         </is>
       </c>
-      <c r="D30" s="35" t="n"/>
-      <c r="E30" s="35" t="n"/>
-      <c r="F30" s="35" t="n"/>
+      <c r="D30" s="53" t="n"/>
+      <c r="E30" s="53" t="n"/>
+      <c r="F30" s="54" t="n"/>
       <c r="G30" s="22" t="n">
         <v>30</v>
       </c>
@@ -1273,9 +1493,9 @@
           <t>Descarga de formularios en PDF/Excel, software, manuales o legislación</t>
         </is>
       </c>
-      <c r="D31" s="33" t="n"/>
-      <c r="E31" s="33" t="n"/>
-      <c r="F31" s="33" t="n"/>
+      <c r="D31" s="53" t="n"/>
+      <c r="E31" s="53" t="n"/>
+      <c r="F31" s="54" t="n"/>
       <c r="G31" s="15" t="n">
         <v>1</v>
       </c>
@@ -1295,9 +1515,9 @@
           <t>100% de contenidos catalogados según interacción digital</t>
         </is>
       </c>
-      <c r="D32" s="24" t="n"/>
-      <c r="E32" s="24" t="n"/>
-      <c r="F32" s="24" t="n"/>
+      <c r="D32" s="53" t="n"/>
+      <c r="E32" s="53" t="n"/>
+      <c r="F32" s="54" t="n"/>
       <c r="G32" s="27">
         <f>SUM(G28:G31)</f>
         <v/>
@@ -3841,4 +4061,1258 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="69" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" s="69" t="inlineStr">
+        <is>
+          <t>Nivel</t>
+        </is>
+      </c>
+      <c r="C1" s="69" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="D1" s="69" t="inlineStr">
+        <is>
+          <t>Qué es</t>
+        </is>
+      </c>
+      <c r="E1" s="69" t="inlineStr">
+        <is>
+          <t>Lead text</t>
+        </is>
+      </c>
+      <c r="F1" s="69" t="inlineStr">
+        <is>
+          <t>Base jurídica</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="C2" s="71" t="inlineStr">
+        <is>
+          <t>Contribuyentes</t>
+        </is>
+      </c>
+      <c r="D2" s="71" t="inlineStr">
+        <is>
+          <t>Son las personas individuales, jurídicas, patrimonios o entes afectos al cumplimiento de obligaciones tributarias internas en el territorio guatemalteco. Abarca a ciudadanos sin actividad económica activa, asalariados en relación de dependencia, pequeños contribuyentes, contribuyentes del régimen general del IVA e ISR, propietarios de vehículos y grandes/medianos contribuyentes especiales calificados.</t>
+        </is>
+      </c>
+      <c r="E2" s="71" t="inlineStr">
+        <is>
+          <t>Información y servicios tributarios para personas y empresas.</t>
+        </is>
+      </c>
+      <c r="F2" s="71" t="inlineStr">
+        <is>
+          <t>Constitución Política (Art. 135d), Código Tributario (Dto. 6-91), Ley del IVA (Dto. 27-92), Ley de Actualización Tributaria (Dto. 10-2012), Ley del ISCV (Dto. 70-94) y Ley de Simplificación Tributaria (Dto. 7-2019 / Dto. 31-2024).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C3" s="71" t="inlineStr">
+        <is>
+          <t>Sin Obligaciones de Impuestos</t>
+        </is>
+      </c>
+      <c r="D3" s="71" t="inlineStr">
+        <is>
+          <t>Personas individuales que no realizan actividades económicas mercantiles pero requieren identificación tributaria para actos civiles, contratos, trámites notariales o apertura de cuentas bancarias.</t>
+        </is>
+      </c>
+      <c r="E3" s="71" t="inlineStr">
+        <is>
+          <t>Obtén tu primer NIT, actualiza tus datos de identificación personal y consulta tu constancia sin movimientos comerciales.</t>
+        </is>
+      </c>
+      <c r="F3" s="71" t="inlineStr">
+        <is>
+          <t>Código Tributario (Decreto 6-91, Arts. 112 y 120), Ley de Actualización Tributaria (Decreto 10-2012) y Acuerdo de Directorio SAT 08-2020.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C4" s="71" t="inlineStr">
+        <is>
+          <t>Asalariados, Compradores de Bienes y Residentes en el Extranjero</t>
+        </is>
+      </c>
+      <c r="D4" s="71" t="inlineStr">
+        <is>
+          <t>Personas individuales que, sin ejercer actividad económica mercantil, tramitan su NIT únicamente para actos civiles, laborales, notariales o bancarios. Agrupa a asalariados sin obligaciones tributarias, compradores de bienes, estudiantes y residentes en el extranjero que requieren identificación tributaria sin declarar impuestos internos.</t>
+        </is>
+      </c>
+      <c r="E4" s="71" t="inlineStr">
+        <is>
+          <t>Solicita tu NIT sin actividad comercial, actualiza tus datos y consulta tus constancias.</t>
+        </is>
+      </c>
+      <c r="F4" s="71" t="inlineStr">
+        <is>
+          <t>Código Tributario (Dto. 6-91, Arts. 112 y 120), Ley de Actualización Tributaria (Dto. 10-2012) y Acuerdo de Directorio SAT 08-2020.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C5" s="71" t="inlineStr">
+        <is>
+          <t>Pequeños Contribuyentes</t>
+        </is>
+      </c>
+      <c r="D5" s="71" t="inlineStr">
+        <is>
+          <t>Régimen tributario simplificado para personas individuales o jurídicas con ventas o servicios de hasta Q150,000 anuales (tarifa definitiva 5% de IVA sin crédito fiscal), así como productores agropecuarios del sector primario.</t>
+        </is>
+      </c>
+      <c r="E5" s="71" t="inlineStr">
+        <is>
+          <t>Facturación electrónica FEL, declaraciones mensuales del 5%, régimen electrónico y facilidades para el sector primario.</t>
+        </is>
+      </c>
+      <c r="F5" s="71" t="inlineStr">
+        <is>
+          <t>Ley del IVA (Decreto 27-92, Arts. 45 al 50), Decreto 7-2019 (Régimen Electrónico) y Decreto 31-2024 (Sector Primario y Agropecuario).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C6" s="71" t="inlineStr">
+        <is>
+          <t>Pequeño Contribuyente General (5% / Régimen Electrónico)</t>
+        </is>
+      </c>
+      <c r="D6" s="71" t="inlineStr">
+        <is>
+          <t>Personas individuales o jurídicas inscritas en el régimen simplificado del IVA del 5% definitivo sobre ingresos brutos, o en el régimen electrónico del Decreto 7-2019, sin derecho a crédito fiscal y con obligación de emitir factura electrónica FEL.</t>
+        </is>
+      </c>
+      <c r="E6" s="71" t="inlineStr">
+        <is>
+          <t>Inscríbete en el régimen del 5%, declara mensualmente y habilita tu facturación FEL.</t>
+        </is>
+      </c>
+      <c r="F6" s="71" t="inlineStr">
+        <is>
+          <t>Ley del IVA (Dto. 27-92, Arts. 45 al 50) y Ley de Simplificación Tributaria (Dto. 7-2019).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C7" s="71" t="inlineStr">
+        <is>
+          <t>Productores del Sector Primario (Régimen Especial)</t>
+        </is>
+      </c>
+      <c r="D7" s="71" t="inlineStr">
+        <is>
+          <t>Productores agropecuarios, silvícolas y pesqueros del sector primario acogidos a regímenes especiales de tributación, incluidos los sujetos al Impuesto de Circulación de Productos (ICT) y los beneficios del Decreto 31-2024.</t>
+        </is>
+      </c>
+      <c r="E7" s="71" t="inlineStr">
+        <is>
+          <t>Regístrate como productor del sector primario y gestiona tu régimen especial e ICT.</t>
+        </is>
+      </c>
+      <c r="F7" s="71" t="inlineStr">
+        <is>
+          <t>Ley del IVA (Dto. 27-92, Arts. 45 al 50), Dto. 31-2024 (Sector Primario y Agropecuario) y Ley del Impuesto de Circulación de Productos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="70" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C8" s="71" t="inlineStr">
+        <is>
+          <t>Régimen General</t>
+        </is>
+      </c>
+      <c r="D8" s="71" t="inlineStr">
+        <is>
+          <t>Personas individuales y jurídicas afectas a las obligaciones tributarias generales del IVA (12%) e ISR (Actividades Lucrativas, Rentas del Capital y del Trabajo), administración del Registro Fiscal de Vehículos, facturación electrónica FEL y solvencia fiscal.</t>
+        </is>
+      </c>
+      <c r="E8" s="71" t="inlineStr">
+        <is>
+          <t>Declaraciones periódicas, facturación digital FEL, RTU Digital, traspasos vehiculares y pago de impuestos.</t>
+        </is>
+      </c>
+      <c r="F8" s="71" t="inlineStr">
+        <is>
+          <t>Código Tributario (Decreto 6-91), Ley del IVA (Decreto 27-92), Ley de Actualización Tributaria (Decreto 10-2012) y Ley del ISCV (Decreto 70-94).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C9" s="71" t="inlineStr">
+        <is>
+          <t>Asalariados y Relación de Dependencia</t>
+        </is>
+      </c>
+      <c r="D9" s="71" t="inlineStr">
+        <is>
+          <t>Trabajadores cuyos ingresos provienen exclusivamente de una relación laboral de dependencia, sujetos a retención mensual de ISR por parte del patrono y a proyección anual con opción de devolución cuando existe retención en exceso.</t>
+        </is>
+      </c>
+      <c r="E9" s="71" t="inlineStr">
+        <is>
+          <t>Consulta tus retenciones de ISR, presenta tu proyección anual y solicita devoluciones como asalariado.</t>
+        </is>
+      </c>
+      <c r="F9" s="71" t="inlineStr">
+        <is>
+          <t>Ley de Actualización Tributaria (Dto. 10-2012, Libro I - ISR Rentas del Trabajo) y su Reglamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="70" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C10" s="71" t="inlineStr">
+        <is>
+          <t>Empresas y Sociedades Mercantiles</t>
+        </is>
+      </c>
+      <c r="D10" s="71" t="inlineStr">
+        <is>
+          <t>Sociedades anónimas, de responsabilidad limitada, sucursales de sociedades extranjeras, contratos asociativos y demás personas jurídicas mercantiles constituidas conforme al Código de Comercio, obligadas a inscribir su RTU, acreditar representantes legales y gestionar su cese o cancelación.</t>
+        </is>
+      </c>
+      <c r="E10" s="71" t="inlineStr">
+        <is>
+          <t>Inscribe tu sociedad, actualiza a sus representantes legales y gestiona su cese o cancelación.</t>
+        </is>
+      </c>
+      <c r="F10" s="71" t="inlineStr">
+        <is>
+          <t>Código de Comercio (Decreto 2-70), Código Tributario (Decreto 6-91, Arts. 112 y 120) y Acuerdo de Directorio SAT 08-2020.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="70" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C11" s="71" t="inlineStr">
+        <is>
+          <t>Contribuyentes Especiales</t>
+        </is>
+      </c>
+      <c r="D11" s="71" t="inlineStr">
+        <is>
+          <t>Grandes y medianos contribuyentes calificados por la SAT con atención gerencial diferenciada, sujetos a fiscalización intensiva, requerimientos de precios de transferencia y presentación de estados financieros auditados.</t>
+        </is>
+      </c>
+      <c r="E11" s="71" t="inlineStr">
+        <is>
+          <t>Atención especializada en gerencias diferenciadas, cumplimiento tributario corporativo y auditorías fiscales.</t>
+        </is>
+      </c>
+      <c r="F11" s="71" t="inlineStr">
+        <is>
+          <t>Ley Orgánica de la SAT (Decreto 1-98, Art. 3) y Resoluciones de Directorio de Calificación de Contribuyentes Especiales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="70" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C12" s="71" t="inlineStr">
+        <is>
+          <t>Grandes y Medianos Contribuyentes</t>
+        </is>
+      </c>
+      <c r="D12" s="71" t="inlineStr">
+        <is>
+          <t>Empresas calificadas mediante Resolución del Directorio como Grandes o Medianos Contribuyentes Especiales, con régimen de atención diferenciada, obligación de reportar operaciones con partes relacionadas (precios de transferencia) y de presentar estados financieros auditados.</t>
+        </is>
+      </c>
+      <c r="E12" s="71" t="inlineStr">
+        <is>
+          <t>Cumple tus obligaciones especiales, presenta estados financieros auditados y gestiona tus estudios de precios de transferencia.</t>
+        </is>
+      </c>
+      <c r="F12" s="71" t="inlineStr">
+        <is>
+          <t>Ley Orgánica de la SAT (Decreto 1-98, Art. 3), Código Tributario (Dto. 6-91, Arts. 112 y 120) y Resoluciones de Directorio sobre Contribuyentes Especiales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="70" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="C13" s="71" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior</t>
+        </is>
+      </c>
+      <c r="D13" s="71" t="inlineStr">
+        <is>
+          <t>Son todas las personas individuales o jurídicas que intervienen en el ingreso, permanencia, traslado y salida de mercancías del territorio aduanero nacional. Comprende tanto a los dueños de las mercancías (importadores y exportadores) como a los prestadores de servicios logísticos autorizados (auxiliares de la función pública, transportistas, depósitos) y empresas que operan bajo regímenes territoriales especiales.</t>
+        </is>
+      </c>
+      <c r="E13" s="71" t="inlineStr">
+        <is>
+          <t>Servicios e información aduanera para la importación, exportación y logística.</t>
+        </is>
+      </c>
+      <c r="F13" s="71" t="inlineStr">
+        <is>
+          <t>Código Tributario (Dto. 6-91), CAUCA IV (Resolución 223-2008 COMIECO) y RECAUCA (Resolución 224-2008 COMIECO).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="70" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C14" s="71" t="inlineStr">
+        <is>
+          <t>Importadores</t>
+        </is>
+      </c>
+      <c r="D14" s="71" t="inlineStr">
+        <is>
+          <t>Personas individuales o jurídicas autorizadas en el padrón aduanero para ingresar legalmente mercancías extranjeras al territorio aduanero nacional para consumo, uso o transformación.</t>
+        </is>
+      </c>
+      <c r="E14" s="71" t="inlineStr">
+        <is>
+          <t>Padrón de importadores, liquidación de declaraciones DUCA-D, despacho aduanero, aranceles e importación vehicular.</t>
+        </is>
+      </c>
+      <c r="F14" s="71" t="inlineStr">
+        <is>
+          <t>CAUCA IV (Arts. 21 y 77), RECAUCA IV (Arts. 317 al 330) y Ley Nacional de Aduanas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="70" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C15" s="71" t="inlineStr">
+        <is>
+          <t>Exportadores</t>
+        </is>
+      </c>
+      <c r="D15" s="71" t="inlineStr">
+        <is>
+          <t>Operadores inscritos en el Registro de Exportadores de la SAT y en la Ventanilla Única para las Exportaciones (VUPE) que despachan mercancías de origen nacional o nacionalizadas hacia mercados extranjeros.</t>
+        </is>
+      </c>
+      <c r="E15" s="71" t="inlineStr">
+        <is>
+          <t>Código VUPE, declaraciones aduaneras de embarque y gestión de devolución de crédito fiscal del IVA.</t>
+        </is>
+      </c>
+      <c r="F15" s="71" t="inlineStr">
+        <is>
+          <t>Ley del IVA (Decreto 27-92, Arts. 23 al 25 bis), Decreto 29-89 (Ley de Maquilas) y CAUCA/RECAUCA IV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="70" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C16" s="71" t="inlineStr">
+        <is>
+          <t>Operador Económico Autorizado (OEA)</t>
+        </is>
+      </c>
+      <c r="D16" s="71" t="inlineStr">
+        <is>
+          <t>Actores de la cadena logística internacional certificados por la SAT con estándares SAFE de la OMA para gozar de despacho preferencial y simplificación aduanera.</t>
+        </is>
+      </c>
+      <c r="E16" s="71" t="inlineStr">
+        <is>
+          <t>Certificación en seguridad logística, carriles exprés y reducción de selectivo rojo en aduanas.</t>
+        </is>
+      </c>
+      <c r="F16" s="71" t="inlineStr">
+        <is>
+          <t>Marco Normativo SAFE de la OMA, CAUCA IV y Resoluciones de Directorio SAT del Programa OEA-Guatemala.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="70" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C17" s="71" t="inlineStr">
+        <is>
+          <t>Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        </is>
+      </c>
+      <c r="D17" s="71" t="inlineStr">
+        <is>
+          <t>Personas naturales o jurídicas autorizadas por la Intendencia de Aduanas para actuar en nombre propio o de terceros en desaduanamiento, transporte, custodia o desconsolidación: agentes aduaneros, apoderados, depósitos temporales, courier y transportistas.</t>
+        </is>
+      </c>
+      <c r="E17" s="71" t="inlineStr">
+        <is>
+          <t>Carnés oficiales, pólizas de fianza operativa, marchamos electrónicos y habilitación de depósitos aduaneros.</t>
+        </is>
+      </c>
+      <c r="F17" s="71" t="inlineStr">
+        <is>
+          <t>CAUCA IV (Arts. 18 al 28), RECAUCA IV (Arts. 74 al 136) y Ley Nacional de Aduanas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="70" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C18" s="71" t="inlineStr">
+        <is>
+          <t>Agentes Aduaneros</t>
+        </is>
+      </c>
+      <c r="D18" s="71" t="inlineStr">
+        <is>
+          <t>Personas naturales autorizadas por la SAT para actuar como auxiliares de la función pública aduanera en el despacho de mercancías por cuenta de importadores y exportadores, con mandato inscrito, fianza vigente y carné oficial.</t>
+        </is>
+      </c>
+      <c r="E18" s="71" t="inlineStr">
+        <is>
+          <t>Inscríbete, renueva tu fianza y actualiza tu carné de agente aduanero.</t>
+        </is>
+      </c>
+      <c r="F18" s="71" t="inlineStr">
+        <is>
+          <t>CAUCA IV (Arts. 22 al 28), RECAUCA IV (Arts. 74 al 85) y Ley Nacional de Aduanas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="70" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C19" s="71" t="inlineStr">
+        <is>
+          <t>Apoderados Especiales Aduaneros</t>
+        </is>
+      </c>
+      <c r="D19" s="71" t="inlineStr">
+        <is>
+          <t>Personas individuales designadas mediante mandato especial por un agente aduanero o por un importador/exportador para realizar operaciones aduaneras determinadas, acreditadas con garantía y carné vigente ante el servicio aduanero.</t>
+        </is>
+      </c>
+      <c r="E19" s="71" t="inlineStr">
+        <is>
+          <t>Habilita tu mandato, acredita tu garantía y gestiona tu carné de apoderado especial aduanero.</t>
+        </is>
+      </c>
+      <c r="F19" s="71" t="inlineStr">
+        <is>
+          <t>CAUCA IV (Arts. 18 al 28) y RECAUCA IV (Arts. 86 al 90, Apoderados Especiales Aduaneros).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="70" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C20" s="71" t="inlineStr">
+        <is>
+          <t>Depósitos Aduaneros</t>
+        </is>
+      </c>
+      <c r="D20" s="71" t="inlineStr">
+        <is>
+          <t>Personas jurídicas autorizadas para almacenar mercancías bajo control aduanero: Depósitos Aduaneros Temporales (DAT), Almacenes Generales de Depósito (AGD) y almacenes fiscales, sujetos a habilitación, garantía y control de inventarios.</t>
+        </is>
+      </c>
+      <c r="E20" s="71" t="inlineStr">
+        <is>
+          <t>Solicita tu habilitación, acredita tu fianza y opera tu depósito aduanero bajo control de la SAT.</t>
+        </is>
+      </c>
+      <c r="F20" s="71" t="inlineStr">
+        <is>
+          <t>Decreto 1236 (Ley de Almacenes Generales de Depósito), RECAUCA IV (Arts. 116 al 130) y CAUCA IV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="70" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C21" s="71" t="inlineStr">
+        <is>
+          <t>Empresas de Entrega Rápida o Courier</t>
+        </is>
+      </c>
+      <c r="D21" s="71" t="inlineStr">
+        <is>
+          <t>Empresas autorizadas para prestar el servicio de entrega rápida o courier, mediante el cual transportan y desaduanan envíos de importación y exportación bajo un régimen aduanero simplificado de despacho.</t>
+        </is>
+      </c>
+      <c r="E21" s="71" t="inlineStr">
+        <is>
+          <t>Habilítate y opera como empresa courier bajo el régimen de envíos de entrega rápida.</t>
+        </is>
+      </c>
+      <c r="F21" s="71" t="inlineStr">
+        <is>
+          <t>CAUCA IV y RECAUCA IV (Arts. 574 al 596, Régimen de Envíos de Entrega Rápida o Courier).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="70" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C22" s="71" t="inlineStr">
+        <is>
+          <t>Transportistas Aduaneros</t>
+        </is>
+      </c>
+      <c r="D22" s="71" t="inlineStr">
+        <is>
+          <t>Empresas de transporte autorizadas para movilizar mercancías hacia recintos aduaneros y en tránsito aduanero, obligadas a operar con manifiestos de carga, marchamo electrónico y equipo habilitado.</t>
+        </is>
+      </c>
+      <c r="E22" s="71" t="inlineStr">
+        <is>
+          <t>Habilita tu flota, gestiona tus manifiestos de carga y opera el marchamo electrónico.</t>
+        </is>
+      </c>
+      <c r="F22" s="71" t="inlineStr">
+        <is>
+          <t>CAUCA IV (Arts. 18 al 28), RECAUCA IV (Tránsito Aduanero Internacional Terrestre) y Ley Nacional de Aduanas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="70" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C23" s="71" t="inlineStr">
+        <is>
+          <t>Regímenes Territoriales y Zonas Especiales</t>
+        </is>
+      </c>
+      <c r="D23" s="71" t="inlineStr">
+        <is>
+          <t>Empresas y parques industriales que operan bajo regímenes aduaneros liberatorios o de fomento con suspensión y exención arancelaria: Maquilas (Decreto 29-89) y Zonas de Desarrollo Económico Especial Público (ZDEEP).</t>
+        </is>
+      </c>
+      <c r="E23" s="71" t="inlineStr">
+        <is>
+          <t>Habilitación ZDEEP, importación con suspensión arancelaria y liquidación de cuentas corrientes bajo el Dto. 29-89.</t>
+        </is>
+      </c>
+      <c r="F23" s="71" t="inlineStr">
+        <is>
+          <t>Decreto 29-89 (Ley de Maquilas), Decreto 22-73 (ZOLIC/ZDEEP) y normativa aduanera aplicable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="70" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C24" s="71" t="inlineStr">
+        <is>
+          <t>Maquilas (Decreto 29-89)</t>
+        </is>
+      </c>
+      <c r="D24" s="71" t="inlineStr">
+        <is>
+          <t>Empresas autorizadas bajo la Ley de Fomento y Desarrollo de la Actividad Exportadora y de Maquila que importan insumos con suspensión de aranceles para transformarlos y exportar el producto final, operando con cuenta corriente y fianza.</t>
+        </is>
+      </c>
+      <c r="E24" s="71" t="inlineStr">
+        <is>
+          <t>Habilita tu empresa maquiladora, administra tu cuenta corriente y libera tu fianza.</t>
+        </is>
+      </c>
+      <c r="F24" s="71" t="inlineStr">
+        <is>
+          <t>Decreto 29-89 (Ley de Fomento y Desarrollo de la Actividad Exportadora y de Maquila) y su Reglamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="70" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C25" s="71" t="inlineStr">
+        <is>
+          <t>Zonas de Desarrollo Económico Especial Público (ZDEEP)</t>
+        </is>
+      </c>
+      <c r="D25" s="71" t="inlineStr">
+        <is>
+          <t>Entidades administradoras y empresas usuarias calificadas que operan dentro de Zonas de Desarrollo Económico Especial Público, con beneficios aduaneros y fiscales para la actividad industrial y de servicios.</t>
+        </is>
+      </c>
+      <c r="E25" s="71" t="inlineStr">
+        <is>
+          <t>Califícate como administrador o empresa usuaria ZDEEP y opera con incentivos bajo control aduanero.</t>
+        </is>
+      </c>
+      <c r="F25" s="71" t="inlineStr">
+        <is>
+          <t>Decreto 22-73 (Ley Orgánica de ZOLIC / ZDEEP), CAUCA IV y RECAUCA IV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="70" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="C26" s="71" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="D26" s="71" t="inlineStr">
+        <is>
+          <t>Son las personas individuales colegiadas activas o técnicos acreditados ante la SAT que ejercen liberalmente su profesión o actúan como auxiliares técnicos en materia tributaria, mercantil y notarial. Comprende a abogados y notarios (traspasos vehiculares electrónicos y fe pública), peritos contadores, contadores públicos y auditores (CPA) y gestores tributarios acreditados.</t>
+        </is>
+      </c>
+      <c r="E26" s="71" t="inlineStr">
+        <is>
+          <t>Herramientas y servicios especializados para profesionales tributarios y auxiliares.</t>
+        </is>
+      </c>
+      <c r="F26" s="71" t="inlineStr">
+        <is>
+          <t>Código de Notariado (Dto. 314), Ley de Colegiación Profesional Obligatoria (Dto. 72-2001), Decreto 2450 (Normas de la Profesión Contable), Ley de Timbres Fiscales (Dto. 37-92) y Código Tributario (Art. 57 "A" y 112).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="70" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C27" s="71" t="inlineStr">
+        <is>
+          <t>Abogados y Notarios</t>
+        </is>
+      </c>
+      <c r="D27" s="71" t="inlineStr">
+        <is>
+          <t>Profesionales del derecho colegiados activos autorizados para la fe pública notarial, venta y razón de timbres fiscales, papel sellado de protocolos y traspasos vehiculares electrónicos (TEV).</t>
+        </is>
+      </c>
+      <c r="E27" s="71" t="inlineStr">
+        <is>
+          <t>Compra de papel de protocolo, razones de timbres, formalización de traspasos en línea TEV y avisos notariales.</t>
+        </is>
+      </c>
+      <c r="F27" s="71" t="inlineStr">
+        <is>
+          <t>Código de Notariado (Decreto 314), Ley de Timbres Fiscales (Decreto 37-92) y Ley del ISCV (Decreto 70-94).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="70" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C28" s="71" t="inlineStr">
+        <is>
+          <t>Peritos Contadores</t>
+        </is>
+      </c>
+      <c r="D28" s="71" t="inlineStr">
+        <is>
+          <t>Técnicos contables acreditados ante la SAT facultados para llevar registros de contabilidad, autorizar libros electrónicos (LET) y firmar declaraciones juradas tributarias.</t>
+        </is>
+      </c>
+      <c r="E28" s="71" t="inlineStr">
+        <is>
+          <t>Registro de contadores, habilitación del Libro Electrónico Tributario (LET) y administración de obligaciones contables.</t>
+        </is>
+      </c>
+      <c r="F28" s="71" t="inlineStr">
+        <is>
+          <t>Decreto 2450 (Normas de la Profesión Contable), Código de Comercio (Arts. 368 al 381) y Código Tributario (Arts. 112 y 120).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="70" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C29" s="71" t="inlineStr">
+        <is>
+          <t>Auditores</t>
+        </is>
+      </c>
+      <c r="D29" s="71" t="inlineStr">
+        <is>
+          <t>Contadores Públicos y Auditores (CPA) colegiados activos facultados para emitir dictámenes periciales de devolución de crédito fiscal a exportadores, auditorías tributarias y estados financieros.</t>
+        </is>
+      </c>
+      <c r="E29" s="71" t="inlineStr">
+        <is>
+          <t>Inscripción registral de firmas de CPA y emisión de dictámenes vinculantes para devolución de crédito fiscal.</t>
+        </is>
+      </c>
+      <c r="F29" s="71" t="inlineStr">
+        <is>
+          <t>Ley de Colegiación Profesional Obligatoria (Decreto 72-2001) y Ley del IVA (Decreto 27-92, Art. 25 bis).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="70" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C30" s="71" t="inlineStr">
+        <is>
+          <t>Gestores Tributarios</t>
+        </is>
+      </c>
+      <c r="D30" s="71" t="inlineStr">
+        <is>
+          <t>Personas autorizadas formalmente con gafete institucional para representar a terceros en la realización presencial de expedientes ante agencias tributarias y aduaneras.</t>
+        </is>
+      </c>
+      <c r="E30" s="71" t="inlineStr">
+        <is>
+          <t>Emisión y renovación de gafetes oficiales de gestor, reposición y consulta del padrón activo institucional.</t>
+        </is>
+      </c>
+      <c r="F30" s="71" t="inlineStr">
+        <is>
+          <t>Código Tributario (Decreto 6-91, Art. 22) y Normativa de Acreditación de Gestores de la SAT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="70" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C31" s="71" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales</t>
+        </is>
+      </c>
+      <c r="D31" s="71" t="inlineStr">
+        <is>
+          <t>Profesionales liberales e independientes que prestan servicios técnicos, científicos, jurídicos o de salud por honorarios, afectos a retenciones del IVA e ISR y actualización registral.</t>
+        </is>
+      </c>
+      <c r="E31" s="71" t="inlineStr">
+        <is>
+          <t>Facturación FEL por honorarios, formularios en Declaraguate, consultas vinculantes y retenciones tributarias.</t>
+        </is>
+      </c>
+      <c r="F31" s="71" t="inlineStr">
+        <is>
+          <t>Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Código Tributario (Arts. 102 al 105).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="70" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="C32" s="71" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="D32" s="71" t="inlineStr">
+        <is>
+          <t>Son las personas jurídicas, entidades del sector público, organismos diplomáticos y organizaciones de la sociedad civil que, por mandato constitucional o ley específica ordinaria, gozan de exención total o parcial de tributos y aranceles en el territorio nacional. Incluye centros educativos, universidades, comunidades religiosas, ONGs, fundaciones sin fines de lucro, municipalidades y ministerios de Estado.</t>
+        </is>
+      </c>
+      <c r="E32" s="71" t="inlineStr">
+        <is>
+          <t>Información y gestiones tributarias para entidades públicas y organizaciones no lucrativas.</t>
+        </is>
+      </c>
+      <c r="F32" s="71" t="inlineStr">
+        <is>
+          <t>Constitución Política (Arts. 37, 73, 88 y 257), Ley de ONGs (Dto. 02-2003), Ley del IVA (Dto. 27-92, Art. 8), Ley de Actualización Tributaria (Dto. 10-2012, Art. 11), Código Municipal (Dto. 12-2002) y Ley Orgánica del Presupuesto (Dto. 101-97).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="70" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C33" s="71" t="inlineStr">
+        <is>
+          <t>Entidades del Estado</t>
+        </is>
+      </c>
+      <c r="D33" s="71" t="inlineStr">
+        <is>
+          <t>Ministerios, secretarías, organismos de Estado, dependencias públicas y entidades descentralizadas que operan como agentes de retención oficial del IVA e ISR y administran parque vehicular institucional.</t>
+        </is>
+      </c>
+      <c r="E33" s="71" t="inlineStr">
+        <is>
+          <t>Unidades ejecutoras en el RTU, constancias de retención en compras públicas y control vehicular oficial.</t>
+        </is>
+      </c>
+      <c r="F33" s="71" t="inlineStr">
+        <is>
+          <t>Ley Orgánica del Presupuesto (Decreto 101-97), Ley del IVA, Ley de Contrataciones del Estado (Decreto 57-92) y Código Tributario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="70" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C34" s="71" t="inlineStr">
+        <is>
+          <t>Constitucionales</t>
+        </is>
+      </c>
+      <c r="D34" s="71" t="inlineStr">
+        <is>
+          <t>Entidades con exención total de tributos reconocida expresamente en la Constitución Política: centros educativos, universidades, comunidades religiosas, misiones diplomáticas y confederaciones deportivas.</t>
+        </is>
+      </c>
+      <c r="E34" s="71" t="inlineStr">
+        <is>
+          <t>Acreditación de exenciones constitucionales, emisión de constancias electrónicas y registro en RTU.</t>
+        </is>
+      </c>
+      <c r="F34" s="71" t="inlineStr">
+        <is>
+          <t>Constitución Política de la República (Arts. 37, 73, 88 y 92), Ley del IVA (Art. 8) y Código Tributario (Art. 62).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="70" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C35" s="71" t="inlineStr">
+        <is>
+          <t>Centros Educativos y Universidades (Arts. 73 y 88)</t>
+        </is>
+      </c>
+      <c r="D35" s="71" t="inlineStr">
+        <is>
+          <t>Centros educativos privados y universidades que gozan de exención del IVA y de otros tributos por mandato de los artículos 73 y 88 de la Constitución, previa acreditación de su personería jurídica y fines educativos ante la SAT.</t>
+        </is>
+      </c>
+      <c r="E35" s="71" t="inlineStr">
+        <is>
+          <t>Acredita tu exención constitucional y obtén tus constancias electrónicas.</t>
+        </is>
+      </c>
+      <c r="F35" s="71" t="inlineStr">
+        <is>
+          <t>Constitución Política de la República (Arts. 73 y 88), Ley del IVA (Dto. 27-92, Art. 8) y Código Tributario (Art. 62).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="70" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C36" s="71" t="inlineStr">
+        <is>
+          <t>Iglesias y Deporte Federado (Arts. 37 y 92)</t>
+        </is>
+      </c>
+      <c r="D36" s="71" t="inlineStr">
+        <is>
+          <t>Comunidades religiosas y entidades del deporte federado que gozan de exención de impuestos conforme a los artículos 37 y 92 de la Constitución, acreditadas mediante personería jurídica y reconocimiento ante la SAT.</t>
+        </is>
+      </c>
+      <c r="E36" s="71" t="inlineStr">
+        <is>
+          <t>Registra tu comunidad religiosa o entidad deportiva y gestiona su exención.</t>
+        </is>
+      </c>
+      <c r="F36" s="71" t="inlineStr">
+        <is>
+          <t>Constitución Política de la República (Arts. 37 y 92), Código Civil (personería jurídica) y Código Tributario (Art. 62).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="70" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C37" s="71" t="inlineStr">
+        <is>
+          <t>No Lucrativos</t>
+        </is>
+      </c>
+      <c r="D37" s="71" t="inlineStr">
+        <is>
+          <t>Organizaciones No Gubernamentales (ONGs), fundaciones benéficas y asociaciones civiles sin fines de lucro con exención formal calificada ante la SAT para fines sociales y de desarrollo.</t>
+        </is>
+      </c>
+      <c r="E37" s="71" t="inlineStr">
+        <is>
+          <t>Solicitud formal de exención de ISR, actualización de directivas en el RTU y constancias tributarias.</t>
+        </is>
+      </c>
+      <c r="F37" s="71" t="inlineStr">
+        <is>
+          <t>Ley de ONGs para el Desarrollo (Decreto 02-2003), Ley de Actualización Tributaria (Decreto 10-2012, Art. 11) y Ley del IVA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="70" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C38" s="71" t="inlineStr">
+        <is>
+          <t>Municipalidades</t>
+        </is>
+      </c>
+      <c r="D38" s="71" t="inlineStr">
+        <is>
+          <t>Las 340 corporaciones municipales autónomas de Guatemala, mancomunidades y empresas municipales prestadoras de servicios públicos comunitarios.</t>
+        </is>
+      </c>
+      <c r="E38" s="71" t="inlineStr">
+        <is>
+          <t>Registro de autoridades y tesoreros en el RTU, solvencias municipales y exención del ISCV para flotillas ediles.</t>
+        </is>
+      </c>
+      <c r="F38" s="71" t="inlineStr">
+        <is>
+          <t>Constitución Política (Art. 257), Código Municipal (Decreto 12-2002) y Ley del ISCV (Decreto 70-94).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="70" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="C39" s="71" t="inlineStr">
+        <is>
+          <t>Decreto</t>
+        </is>
+      </c>
+      <c r="D39" s="71" t="inlineStr">
+        <is>
+          <t>Entidades beneficiarias de incentivos y exenciones tributarias específicas aprobadas mediante decretos legislativos ordinarios del Congreso: cooperativas, partidos políticos, donaciones oficiales y fomento sectorial.</t>
+        </is>
+      </c>
+      <c r="E39" s="71" t="inlineStr">
+        <is>
+          <t>Gestión de exenciones por ley ordinaria, despacho aduanero de donaciones y constancias oficiales.</t>
+        </is>
+      </c>
+      <c r="F39" s="71" t="inlineStr">
+        <is>
+          <t>Ley General de Cooperativas (Decreto 82-78), Ley Electoral y de Partidos Políticos (Decreto 1-85) y decretos de fomento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="70" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C40" s="71" t="inlineStr">
+        <is>
+          <t>Cooperativas, Partidos Políticos y Exenciones Especiales</t>
+        </is>
+      </c>
+      <c r="D40" s="71" t="inlineStr">
+        <is>
+          <t>Cooperativas, partidos políticos y otras entidades beneficiarias de exenciones tributarias otorgadas por leyes ordinarias, sujetas a reconocimiento y control de vigencia ante la SAT.</t>
+        </is>
+      </c>
+      <c r="E40" s="71" t="inlineStr">
+        <is>
+          <t>Gestiona la exención por ley especial de tu cooperativa, partido político o entidad.</t>
+        </is>
+      </c>
+      <c r="F40" s="71" t="inlineStr">
+        <is>
+          <t>Ley General de Cooperativas (Dto. 82-78), Ley Electoral y de Partidos Políticos (Dto. 1-85) y decretos de exención específicos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="70" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="70" t="inlineStr">
+        <is>
+          <t>Nivel 3</t>
+        </is>
+      </c>
+      <c r="C41" s="71" t="inlineStr">
+        <is>
+          <t>Misiones Diplomáticas y Organismos Internacionales</t>
+        </is>
+      </c>
+      <c r="D41" s="71" t="inlineStr">
+        <is>
+          <t>Representaciones diplomáticas, consulares y organismos internacionales acreditados en Guatemala que solicitan el reconocimiento de sus exenciones tributarias conforme al derecho internacional y a los convenios de sede vigentes.</t>
+        </is>
+      </c>
+      <c r="E41" s="71" t="inlineStr">
+        <is>
+          <t>Solicita el reconocimiento de exenciones y gestiona tus constancias como misión u organismo acreditado.</t>
+        </is>
+      </c>
+      <c r="F41" s="71" t="inlineStr">
+        <is>
+          <t>Convención de Viena sobre Relaciones Diplomáticas (1961), convenios de sede suscritos por Guatemala y Código Tributario (Art. 62).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(taxonomy): compactar N3/N4/N5 en Pequeños Contribuyentes y corregir SAT-GES-0012
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -987,7 +987,7 @@
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ARQUITECTURA DE INFORMACIÓN DEL PORTAL WEB — DEFINICIÓN DE SEGMENTOS, LEAD TEXT Y BASE JURÍDICA</t>
+          <t>ARQUITECTURA DE INFORMACIÓN DEL PORTAL WEB — DEFINICIÓN DE NIVEL 1, LEAD TEXT Y BASE JURÍDICA</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
     <row r="9">
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>1. SEGMENTOS PRINCIPALES DEL PORTAL (NIVEL 1) — DEFINICIONES INSTITUCIONALES</t>
+          <t>1. NIVEL 1 — DEFINICIONES INSTITUCIONALES</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Segmento (Nivel 1)</t>
+          <t>Nivel 1</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Nivel 1: Segmento Oficial</t>
+          <t>Nivel 1</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Nivel 2: Régimen / Área</t>
+          <t>Nivel 2</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Nivel 3: Categoría / Actor</t>
+          <t>Nivel 3</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>% Segmento</t>
+          <t>% Nivel 1</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D18" s="44" t="inlineStr">
         <is>
-          <t>11 Categorías / Actores</t>
+          <t>11 nodos de Nivel 3</t>
         </is>
       </c>
       <c r="E18" s="42" t="inlineStr"/>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="D25" s="44" t="inlineStr">
         <is>
-          <t>6 Categorías / Actores</t>
+          <t>6 nodos de Nivel 3</t>
         </is>
       </c>
       <c r="E25" s="42" t="inlineStr"/>
@@ -2613,7 +2613,7 @@
       </c>
       <c r="D31" s="44" t="inlineStr">
         <is>
-          <t>5 Categorías / Actores</t>
+          <t>5 nodos de Nivel 3</t>
         </is>
       </c>
       <c r="E31" s="42" t="inlineStr"/>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="D37" s="44" t="inlineStr">
         <is>
-          <t>5 Categorías / Actores</t>
+          <t>5 nodos de Nivel 3</t>
         </is>
       </c>
       <c r="E37" s="42" t="inlineStr"/>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="D38" s="49" t="inlineStr">
         <is>
-          <t>4 Segmentos y 27 Categorías</t>
+          <t>4 nodos de Nivel 1 y 27 nodos de Nivel 3</t>
         </is>
       </c>
       <c r="E38" s="47" t="inlineStr"/>
@@ -2952,7 +2952,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MATRIZ COMPLETA DE LAS 27 CATEGORÍAS DEL PORTAL CON SUS TEXTOS ORIENTADORES Y MARCO NORMATIVO OFICIAL</t>
+          <t>MATRIZ COMPLETA DE LOS 27 NODOS DE NIVEL 3 DEL PORTAL CON SUS TEXTOS ORIENTADORES Y MARCO NORMATIVO OFICIAL</t>
         </is>
       </c>
     </row>
@@ -2964,17 +2964,17 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Segmento (Nivel 1)</t>
+          <t>Nivel 1</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Régimen / Área (Nivel 2)</t>
+          <t>Nivel 2</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Categoría / Actor (Nivel 3)</t>
+          <t>Nivel 3</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -4033,12 +4033,12 @@
       </c>
       <c r="C34" s="49" t="inlineStr">
         <is>
-          <t>4 Segmentos Oficiales</t>
+          <t>4 nodos de Nivel 1</t>
         </is>
       </c>
       <c r="D34" s="49" t="inlineStr">
         <is>
-          <t>27 Categorías</t>
+          <t>27 nodos de Nivel 3</t>
         </is>
       </c>
       <c r="E34" s="49" t="inlineStr">

</xml_diff>

<commit_message>
feat(ia): auditar arquitectura de informacion, compactar N5 y sincronizar documentacion
- Optimizar profundidad del catalogo reduciendo N5 de 111 a 70 tramites
- Compactar nodos pasarela en Contribuyentes Especiales y Municipalidades
- Sincronizar matriz viva de 715 tramites en Excel, JSON y contratos TypeScript
- Normalizar rotulos estrictamente numericos (N1-N5) erradicando nombres conceptuales
- Completar metadatos en Entes Exentos (100%) y limpiar numeros quemados en titulos
- Actualizar y validar documentacion en docs/, database/ y componentes UI
- 20/20 pruebas Playwright exitosas con 0 violaciones WCAG 2.2 AA
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -10,7 +10,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen Arquitectura" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa de Navegación" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fichas por Rol y Categoría" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fichas por Nivel" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fichas por Rol y Categoría'!$A$6:$H$33</definedName>
@@ -24,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,28 +95,8 @@
       <color rgb="001E293B"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="000F172A"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="17">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -178,38 +157,8 @@
         <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0019324B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0014649B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DCE6F1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EDF3FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2E8F0"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="18">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -303,127 +252,11 @@
         <color rgb="0064748B"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B7C3D0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00B7C3D0"/>
-      </right>
-      <top style="medium">
-        <color rgb="0014649B"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="0014649B"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B7C3D0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00B7C3D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B7C3D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00B7C3D0"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="0014649B"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00B7C3D0"/>
-      </right>
-      <top style="medium">
-        <color rgb="0014649B"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="0014649B"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="0014649B"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00B7C3D0"/>
-      </right>
-      <top style="medium">
-        <color rgb="0014649B"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="0014649B"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -544,59 +377,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1262,11 +1042,11 @@
           <t>Primer NIT, RTU Digital, padrones de importación/exportación y habilitación inicial</t>
         </is>
       </c>
-      <c r="D19" s="53" t="n"/>
-      <c r="E19" s="53" t="n"/>
-      <c r="F19" s="54" t="n"/>
+      <c r="D19" s="33" t="n"/>
+      <c r="E19" s="33" t="n"/>
+      <c r="F19" s="33" t="n"/>
       <c r="G19" s="15" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="H19" s="16">
         <f>G19/$G$24</f>
@@ -1284,9 +1064,9 @@
           <t>Facturación FEL, Declaraguate, DUCAs, retenciones, transferencias y pagos</t>
         </is>
       </c>
-      <c r="D20" s="53" t="n"/>
-      <c r="E20" s="53" t="n"/>
-      <c r="F20" s="54" t="n"/>
+      <c r="D20" s="35" t="n"/>
+      <c r="E20" s="35" t="n"/>
+      <c r="F20" s="35" t="n"/>
       <c r="G20" s="22" t="n">
         <v>260</v>
       </c>
@@ -1306,9 +1086,9 @@
           <t>Verificadores en tiempo real, solvencia, selectivo aduanero, rampa y SAC</t>
         </is>
       </c>
-      <c r="D21" s="53" t="n"/>
-      <c r="E21" s="53" t="n"/>
-      <c r="F21" s="54" t="n"/>
+      <c r="D21" s="33" t="n"/>
+      <c r="E21" s="33" t="n"/>
+      <c r="F21" s="33" t="n"/>
       <c r="G21" s="15" t="n">
         <v>116</v>
       </c>
@@ -1328,11 +1108,11 @@
           <t>Actualización de RTU, traspaso vehicular, prórrogas, cese de actividades y subastas</t>
         </is>
       </c>
-      <c r="D22" s="53" t="n"/>
-      <c r="E22" s="53" t="n"/>
-      <c r="F22" s="54" t="n"/>
+      <c r="D22" s="35" t="n"/>
+      <c r="E22" s="35" t="n"/>
+      <c r="F22" s="35" t="n"/>
       <c r="G22" s="22" t="n">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="H22" s="23">
         <f>G22/$G$24</f>
@@ -1350,9 +1130,9 @@
           <t>Marco legal aduanero y tributario, devoluciones, criterios institucionales y cursos</t>
         </is>
       </c>
-      <c r="D23" s="53" t="n"/>
-      <c r="E23" s="53" t="n"/>
-      <c r="F23" s="54" t="n"/>
+      <c r="D23" s="33" t="n"/>
+      <c r="E23" s="33" t="n"/>
+      <c r="F23" s="33" t="n"/>
       <c r="G23" s="15" t="n">
         <v>130</v>
       </c>
@@ -1372,9 +1152,9 @@
           <t>100% de contenidos clasificados según ciclo de vida</t>
         </is>
       </c>
-      <c r="D24" s="53" t="n"/>
-      <c r="E24" s="53" t="n"/>
-      <c r="F24" s="54" t="n"/>
+      <c r="D24" s="24" t="n"/>
+      <c r="E24" s="24" t="n"/>
+      <c r="F24" s="24" t="n"/>
       <c r="G24" s="27">
         <f>SUM(G19:G23)</f>
         <v/>
@@ -1427,9 +1207,9 @@
           <t>Páginas explicativas, requisitos de trámites presenciales o mixtos</t>
         </is>
       </c>
-      <c r="D28" s="53" t="n"/>
-      <c r="E28" s="53" t="n"/>
-      <c r="F28" s="54" t="n"/>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="35" t="n"/>
+      <c r="F28" s="35" t="n"/>
       <c r="G28" s="22" t="n">
         <v>490</v>
       </c>
@@ -1449,9 +1229,9 @@
           <t>Servicios digitales transaccionales (Agencia Virtual, Declaraguate, TEV, FEL)</t>
         </is>
       </c>
-      <c r="D29" s="53" t="n"/>
-      <c r="E29" s="53" t="n"/>
-      <c r="F29" s="54" t="n"/>
+      <c r="D29" s="33" t="n"/>
+      <c r="E29" s="33" t="n"/>
+      <c r="F29" s="33" t="n"/>
       <c r="G29" s="15" t="n">
         <v>137</v>
       </c>
@@ -1471,11 +1251,11 @@
           <t>Herramientas de verificación sin autenticación previa (RTU público, solvencias)</t>
         </is>
       </c>
-      <c r="D30" s="53" t="n"/>
-      <c r="E30" s="53" t="n"/>
-      <c r="F30" s="54" t="n"/>
+      <c r="D30" s="35" t="n"/>
+      <c r="E30" s="35" t="n"/>
+      <c r="F30" s="35" t="n"/>
       <c r="G30" s="22" t="n">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="H30" s="23">
         <f>G30/$G$32</f>
@@ -1493,11 +1273,11 @@
           <t>Descarga de formularios en PDF/Excel, software, manuales o legislación</t>
         </is>
       </c>
-      <c r="D31" s="53" t="n"/>
-      <c r="E31" s="53" t="n"/>
-      <c r="F31" s="54" t="n"/>
+      <c r="D31" s="33" t="n"/>
+      <c r="E31" s="33" t="n"/>
+      <c r="F31" s="33" t="n"/>
       <c r="G31" s="15" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="H31" s="16">
         <f>G31/$G$32</f>
@@ -1515,9 +1295,9 @@
           <t>100% de contenidos catalogados según interacción digital</t>
         </is>
       </c>
-      <c r="D32" s="53" t="n"/>
-      <c r="E32" s="53" t="n"/>
-      <c r="F32" s="54" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="24" t="n"/>
       <c r="G32" s="27">
         <f>SUM(G28:G31)</f>
         <v/>
@@ -1661,7 +1441,7 @@
         </is>
       </c>
       <c r="G7" s="15" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H7" s="38">
         <f>G7/$G$18</f>
@@ -3033,7 +2813,7 @@
         </is>
       </c>
       <c r="H7" s="15" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="54" customHeight="1">
@@ -4061,1258 +3841,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="58" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="69" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B1" s="69" t="inlineStr">
-        <is>
-          <t>Nivel</t>
-        </is>
-      </c>
-      <c r="C1" s="69" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="D1" s="69" t="inlineStr">
-        <is>
-          <t>Qué es</t>
-        </is>
-      </c>
-      <c r="E1" s="69" t="inlineStr">
-        <is>
-          <t>Lead text</t>
-        </is>
-      </c>
-      <c r="F1" s="69" t="inlineStr">
-        <is>
-          <t>Base jurídica</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 1</t>
-        </is>
-      </c>
-      <c r="C2" s="71" t="inlineStr">
-        <is>
-          <t>Contribuyentes</t>
-        </is>
-      </c>
-      <c r="D2" s="71" t="inlineStr">
-        <is>
-          <t>Son las personas individuales, jurídicas, patrimonios o entes afectos al cumplimiento de obligaciones tributarias internas en el territorio guatemalteco. Abarca a ciudadanos sin actividad económica activa, asalariados en relación de dependencia, pequeños contribuyentes, contribuyentes del régimen general del IVA e ISR, propietarios de vehículos y grandes/medianos contribuyentes especiales calificados.</t>
-        </is>
-      </c>
-      <c r="E2" s="71" t="inlineStr">
-        <is>
-          <t>Información y servicios tributarios para personas y empresas.</t>
-        </is>
-      </c>
-      <c r="F2" s="71" t="inlineStr">
-        <is>
-          <t>Constitución Política (Art. 135d), Código Tributario (Dto. 6-91), Ley del IVA (Dto. 27-92), Ley de Actualización Tributaria (Dto. 10-2012), Ley del ISCV (Dto. 70-94) y Ley de Simplificación Tributaria (Dto. 7-2019 / Dto. 31-2024).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C3" s="71" t="inlineStr">
-        <is>
-          <t>Sin Obligaciones de Impuestos</t>
-        </is>
-      </c>
-      <c r="D3" s="71" t="inlineStr">
-        <is>
-          <t>Personas individuales que no realizan actividades económicas mercantiles pero requieren identificación tributaria para actos civiles, contratos, trámites notariales o apertura de cuentas bancarias.</t>
-        </is>
-      </c>
-      <c r="E3" s="71" t="inlineStr">
-        <is>
-          <t>Obtén tu primer NIT, actualiza tus datos de identificación personal y consulta tu constancia sin movimientos comerciales.</t>
-        </is>
-      </c>
-      <c r="F3" s="71" t="inlineStr">
-        <is>
-          <t>Código Tributario (Decreto 6-91, Arts. 112 y 120), Ley de Actualización Tributaria (Decreto 10-2012) y Acuerdo de Directorio SAT 08-2020.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C4" s="71" t="inlineStr">
-        <is>
-          <t>Asalariados, Compradores de Bienes y Residentes en el Extranjero</t>
-        </is>
-      </c>
-      <c r="D4" s="71" t="inlineStr">
-        <is>
-          <t>Personas individuales que, sin ejercer actividad económica mercantil, tramitan su NIT únicamente para actos civiles, laborales, notariales o bancarios. Agrupa a asalariados sin obligaciones tributarias, compradores de bienes, estudiantes y residentes en el extranjero que requieren identificación tributaria sin declarar impuestos internos.</t>
-        </is>
-      </c>
-      <c r="E4" s="71" t="inlineStr">
-        <is>
-          <t>Solicita tu NIT sin actividad comercial, actualiza tus datos y consulta tus constancias.</t>
-        </is>
-      </c>
-      <c r="F4" s="71" t="inlineStr">
-        <is>
-          <t>Código Tributario (Dto. 6-91, Arts. 112 y 120), Ley de Actualización Tributaria (Dto. 10-2012) y Acuerdo de Directorio SAT 08-2020.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C5" s="71" t="inlineStr">
-        <is>
-          <t>Pequeños Contribuyentes</t>
-        </is>
-      </c>
-      <c r="D5" s="71" t="inlineStr">
-        <is>
-          <t>Régimen tributario simplificado para personas individuales o jurídicas con ventas o servicios de hasta Q150,000 anuales (tarifa definitiva 5% de IVA sin crédito fiscal), así como productores agropecuarios del sector primario.</t>
-        </is>
-      </c>
-      <c r="E5" s="71" t="inlineStr">
-        <is>
-          <t>Facturación electrónica FEL, declaraciones mensuales del 5%, régimen electrónico y facilidades para el sector primario.</t>
-        </is>
-      </c>
-      <c r="F5" s="71" t="inlineStr">
-        <is>
-          <t>Ley del IVA (Decreto 27-92, Arts. 45 al 50), Decreto 7-2019 (Régimen Electrónico) y Decreto 31-2024 (Sector Primario y Agropecuario).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C6" s="71" t="inlineStr">
-        <is>
-          <t>Pequeño Contribuyente General (5% / Régimen Electrónico)</t>
-        </is>
-      </c>
-      <c r="D6" s="71" t="inlineStr">
-        <is>
-          <t>Personas individuales o jurídicas inscritas en el régimen simplificado del IVA del 5% definitivo sobre ingresos brutos, o en el régimen electrónico del Decreto 7-2019, sin derecho a crédito fiscal y con obligación de emitir factura electrónica FEL.</t>
-        </is>
-      </c>
-      <c r="E6" s="71" t="inlineStr">
-        <is>
-          <t>Inscríbete en el régimen del 5%, declara mensualmente y habilita tu facturación FEL.</t>
-        </is>
-      </c>
-      <c r="F6" s="71" t="inlineStr">
-        <is>
-          <t>Ley del IVA (Dto. 27-92, Arts. 45 al 50) y Ley de Simplificación Tributaria (Dto. 7-2019).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="70" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C7" s="71" t="inlineStr">
-        <is>
-          <t>Productores del Sector Primario (Régimen Especial)</t>
-        </is>
-      </c>
-      <c r="D7" s="71" t="inlineStr">
-        <is>
-          <t>Productores agropecuarios, silvícolas y pesqueros del sector primario acogidos a regímenes especiales de tributación, incluidos los sujetos al Impuesto de Circulación de Productos (ICT) y los beneficios del Decreto 31-2024.</t>
-        </is>
-      </c>
-      <c r="E7" s="71" t="inlineStr">
-        <is>
-          <t>Regístrate como productor del sector primario y gestiona tu régimen especial e ICT.</t>
-        </is>
-      </c>
-      <c r="F7" s="71" t="inlineStr">
-        <is>
-          <t>Ley del IVA (Dto. 27-92, Arts. 45 al 50), Dto. 31-2024 (Sector Primario y Agropecuario) y Ley del Impuesto de Circulación de Productos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C8" s="71" t="inlineStr">
-        <is>
-          <t>Régimen General</t>
-        </is>
-      </c>
-      <c r="D8" s="71" t="inlineStr">
-        <is>
-          <t>Personas individuales y jurídicas afectas a las obligaciones tributarias generales del IVA (12%) e ISR (Actividades Lucrativas, Rentas del Capital y del Trabajo), administración del Registro Fiscal de Vehículos, facturación electrónica FEL y solvencia fiscal.</t>
-        </is>
-      </c>
-      <c r="E8" s="71" t="inlineStr">
-        <is>
-          <t>Declaraciones periódicas, facturación digital FEL, RTU Digital, traspasos vehiculares y pago de impuestos.</t>
-        </is>
-      </c>
-      <c r="F8" s="71" t="inlineStr">
-        <is>
-          <t>Código Tributario (Decreto 6-91), Ley del IVA (Decreto 27-92), Ley de Actualización Tributaria (Decreto 10-2012) y Ley del ISCV (Decreto 70-94).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C9" s="71" t="inlineStr">
-        <is>
-          <t>Asalariados y Relación de Dependencia</t>
-        </is>
-      </c>
-      <c r="D9" s="71" t="inlineStr">
-        <is>
-          <t>Trabajadores cuyos ingresos provienen exclusivamente de una relación laboral de dependencia, sujetos a retención mensual de ISR por parte del patrono y a proyección anual con opción de devolución cuando existe retención en exceso.</t>
-        </is>
-      </c>
-      <c r="E9" s="71" t="inlineStr">
-        <is>
-          <t>Consulta tus retenciones de ISR, presenta tu proyección anual y solicita devoluciones como asalariado.</t>
-        </is>
-      </c>
-      <c r="F9" s="71" t="inlineStr">
-        <is>
-          <t>Ley de Actualización Tributaria (Dto. 10-2012, Libro I - ISR Rentas del Trabajo) y su Reglamento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="70" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C10" s="71" t="inlineStr">
-        <is>
-          <t>Empresas y Sociedades Mercantiles</t>
-        </is>
-      </c>
-      <c r="D10" s="71" t="inlineStr">
-        <is>
-          <t>Sociedades anónimas, de responsabilidad limitada, sucursales de sociedades extranjeras, contratos asociativos y demás personas jurídicas mercantiles constituidas conforme al Código de Comercio, obligadas a inscribir su RTU, acreditar representantes legales y gestionar su cese o cancelación.</t>
-        </is>
-      </c>
-      <c r="E10" s="71" t="inlineStr">
-        <is>
-          <t>Inscribe tu sociedad, actualiza a sus representantes legales y gestiona su cese o cancelación.</t>
-        </is>
-      </c>
-      <c r="F10" s="71" t="inlineStr">
-        <is>
-          <t>Código de Comercio (Decreto 2-70), Código Tributario (Decreto 6-91, Arts. 112 y 120) y Acuerdo de Directorio SAT 08-2020.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="70" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C11" s="71" t="inlineStr">
-        <is>
-          <t>Contribuyentes Especiales</t>
-        </is>
-      </c>
-      <c r="D11" s="71" t="inlineStr">
-        <is>
-          <t>Grandes y medianos contribuyentes calificados por la SAT con atención gerencial diferenciada, sujetos a fiscalización intensiva, requerimientos de precios de transferencia y presentación de estados financieros auditados.</t>
-        </is>
-      </c>
-      <c r="E11" s="71" t="inlineStr">
-        <is>
-          <t>Atención especializada en gerencias diferenciadas, cumplimiento tributario corporativo y auditorías fiscales.</t>
-        </is>
-      </c>
-      <c r="F11" s="71" t="inlineStr">
-        <is>
-          <t>Ley Orgánica de la SAT (Decreto 1-98, Art. 3) y Resoluciones de Directorio de Calificación de Contribuyentes Especiales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="70" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C12" s="71" t="inlineStr">
-        <is>
-          <t>Grandes y Medianos Contribuyentes</t>
-        </is>
-      </c>
-      <c r="D12" s="71" t="inlineStr">
-        <is>
-          <t>Empresas calificadas mediante Resolución del Directorio como Grandes o Medianos Contribuyentes Especiales, con régimen de atención diferenciada, obligación de reportar operaciones con partes relacionadas (precios de transferencia) y de presentar estados financieros auditados.</t>
-        </is>
-      </c>
-      <c r="E12" s="71" t="inlineStr">
-        <is>
-          <t>Cumple tus obligaciones especiales, presenta estados financieros auditados y gestiona tus estudios de precios de transferencia.</t>
-        </is>
-      </c>
-      <c r="F12" s="71" t="inlineStr">
-        <is>
-          <t>Ley Orgánica de la SAT (Decreto 1-98, Art. 3), Código Tributario (Dto. 6-91, Arts. 112 y 120) y Resoluciones de Directorio sobre Contribuyentes Especiales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="70" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 1</t>
-        </is>
-      </c>
-      <c r="C13" s="71" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D13" s="71" t="inlineStr">
-        <is>
-          <t>Son todas las personas individuales o jurídicas que intervienen en el ingreso, permanencia, traslado y salida de mercancías del territorio aduanero nacional. Comprende tanto a los dueños de las mercancías (importadores y exportadores) como a los prestadores de servicios logísticos autorizados (auxiliares de la función pública, transportistas, depósitos) y empresas que operan bajo regímenes territoriales especiales.</t>
-        </is>
-      </c>
-      <c r="E13" s="71" t="inlineStr">
-        <is>
-          <t>Servicios e información aduanera para la importación, exportación y logística.</t>
-        </is>
-      </c>
-      <c r="F13" s="71" t="inlineStr">
-        <is>
-          <t>Código Tributario (Dto. 6-91), CAUCA IV (Resolución 223-2008 COMIECO) y RECAUCA (Resolución 224-2008 COMIECO).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="70" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C14" s="71" t="inlineStr">
-        <is>
-          <t>Importadores</t>
-        </is>
-      </c>
-      <c r="D14" s="71" t="inlineStr">
-        <is>
-          <t>Personas individuales o jurídicas autorizadas en el padrón aduanero para ingresar legalmente mercancías extranjeras al territorio aduanero nacional para consumo, uso o transformación.</t>
-        </is>
-      </c>
-      <c r="E14" s="71" t="inlineStr">
-        <is>
-          <t>Padrón de importadores, liquidación de declaraciones DUCA-D, despacho aduanero, aranceles e importación vehicular.</t>
-        </is>
-      </c>
-      <c r="F14" s="71" t="inlineStr">
-        <is>
-          <t>CAUCA IV (Arts. 21 y 77), RECAUCA IV (Arts. 317 al 330) y Ley Nacional de Aduanas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="70" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C15" s="71" t="inlineStr">
-        <is>
-          <t>Exportadores</t>
-        </is>
-      </c>
-      <c r="D15" s="71" t="inlineStr">
-        <is>
-          <t>Operadores inscritos en el Registro de Exportadores de la SAT y en la Ventanilla Única para las Exportaciones (VUPE) que despachan mercancías de origen nacional o nacionalizadas hacia mercados extranjeros.</t>
-        </is>
-      </c>
-      <c r="E15" s="71" t="inlineStr">
-        <is>
-          <t>Código VUPE, declaraciones aduaneras de embarque y gestión de devolución de crédito fiscal del IVA.</t>
-        </is>
-      </c>
-      <c r="F15" s="71" t="inlineStr">
-        <is>
-          <t>Ley del IVA (Decreto 27-92, Arts. 23 al 25 bis), Decreto 29-89 (Ley de Maquilas) y CAUCA/RECAUCA IV.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="70" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C16" s="71" t="inlineStr">
-        <is>
-          <t>Operador Económico Autorizado (OEA)</t>
-        </is>
-      </c>
-      <c r="D16" s="71" t="inlineStr">
-        <is>
-          <t>Actores de la cadena logística internacional certificados por la SAT con estándares SAFE de la OMA para gozar de despacho preferencial y simplificación aduanera.</t>
-        </is>
-      </c>
-      <c r="E16" s="71" t="inlineStr">
-        <is>
-          <t>Certificación en seguridad logística, carriles exprés y reducción de selectivo rojo en aduanas.</t>
-        </is>
-      </c>
-      <c r="F16" s="71" t="inlineStr">
-        <is>
-          <t>Marco Normativo SAFE de la OMA, CAUCA IV y Resoluciones de Directorio SAT del Programa OEA-Guatemala.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="70" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C17" s="71" t="inlineStr">
-        <is>
-          <t>Auxiliares de la Función Pública Aduanera (AFPA)</t>
-        </is>
-      </c>
-      <c r="D17" s="71" t="inlineStr">
-        <is>
-          <t>Personas naturales o jurídicas autorizadas por la Intendencia de Aduanas para actuar en nombre propio o de terceros en desaduanamiento, transporte, custodia o desconsolidación: agentes aduaneros, apoderados, depósitos temporales, courier y transportistas.</t>
-        </is>
-      </c>
-      <c r="E17" s="71" t="inlineStr">
-        <is>
-          <t>Carnés oficiales, pólizas de fianza operativa, marchamos electrónicos y habilitación de depósitos aduaneros.</t>
-        </is>
-      </c>
-      <c r="F17" s="71" t="inlineStr">
-        <is>
-          <t>CAUCA IV (Arts. 18 al 28), RECAUCA IV (Arts. 74 al 136) y Ley Nacional de Aduanas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="70" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C18" s="71" t="inlineStr">
-        <is>
-          <t>Agentes Aduaneros</t>
-        </is>
-      </c>
-      <c r="D18" s="71" t="inlineStr">
-        <is>
-          <t>Personas naturales autorizadas por la SAT para actuar como auxiliares de la función pública aduanera en el despacho de mercancías por cuenta de importadores y exportadores, con mandato inscrito, fianza vigente y carné oficial.</t>
-        </is>
-      </c>
-      <c r="E18" s="71" t="inlineStr">
-        <is>
-          <t>Inscríbete, renueva tu fianza y actualiza tu carné de agente aduanero.</t>
-        </is>
-      </c>
-      <c r="F18" s="71" t="inlineStr">
-        <is>
-          <t>CAUCA IV (Arts. 22 al 28), RECAUCA IV (Arts. 74 al 85) y Ley Nacional de Aduanas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="70" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C19" s="71" t="inlineStr">
-        <is>
-          <t>Apoderados Especiales Aduaneros</t>
-        </is>
-      </c>
-      <c r="D19" s="71" t="inlineStr">
-        <is>
-          <t>Personas individuales designadas mediante mandato especial por un agente aduanero o por un importador/exportador para realizar operaciones aduaneras determinadas, acreditadas con garantía y carné vigente ante el servicio aduanero.</t>
-        </is>
-      </c>
-      <c r="E19" s="71" t="inlineStr">
-        <is>
-          <t>Habilita tu mandato, acredita tu garantía y gestiona tu carné de apoderado especial aduanero.</t>
-        </is>
-      </c>
-      <c r="F19" s="71" t="inlineStr">
-        <is>
-          <t>CAUCA IV (Arts. 18 al 28) y RECAUCA IV (Arts. 86 al 90, Apoderados Especiales Aduaneros).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="70" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C20" s="71" t="inlineStr">
-        <is>
-          <t>Depósitos Aduaneros</t>
-        </is>
-      </c>
-      <c r="D20" s="71" t="inlineStr">
-        <is>
-          <t>Personas jurídicas autorizadas para almacenar mercancías bajo control aduanero: Depósitos Aduaneros Temporales (DAT), Almacenes Generales de Depósito (AGD) y almacenes fiscales, sujetos a habilitación, garantía y control de inventarios.</t>
-        </is>
-      </c>
-      <c r="E20" s="71" t="inlineStr">
-        <is>
-          <t>Solicita tu habilitación, acredita tu fianza y opera tu depósito aduanero bajo control de la SAT.</t>
-        </is>
-      </c>
-      <c r="F20" s="71" t="inlineStr">
-        <is>
-          <t>Decreto 1236 (Ley de Almacenes Generales de Depósito), RECAUCA IV (Arts. 116 al 130) y CAUCA IV.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="70" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C21" s="71" t="inlineStr">
-        <is>
-          <t>Empresas de Entrega Rápida o Courier</t>
-        </is>
-      </c>
-      <c r="D21" s="71" t="inlineStr">
-        <is>
-          <t>Empresas autorizadas para prestar el servicio de entrega rápida o courier, mediante el cual transportan y desaduanan envíos de importación y exportación bajo un régimen aduanero simplificado de despacho.</t>
-        </is>
-      </c>
-      <c r="E21" s="71" t="inlineStr">
-        <is>
-          <t>Habilítate y opera como empresa courier bajo el régimen de envíos de entrega rápida.</t>
-        </is>
-      </c>
-      <c r="F21" s="71" t="inlineStr">
-        <is>
-          <t>CAUCA IV y RECAUCA IV (Arts. 574 al 596, Régimen de Envíos de Entrega Rápida o Courier).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="70" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C22" s="71" t="inlineStr">
-        <is>
-          <t>Transportistas Aduaneros</t>
-        </is>
-      </c>
-      <c r="D22" s="71" t="inlineStr">
-        <is>
-          <t>Empresas de transporte autorizadas para movilizar mercancías hacia recintos aduaneros y en tránsito aduanero, obligadas a operar con manifiestos de carga, marchamo electrónico y equipo habilitado.</t>
-        </is>
-      </c>
-      <c r="E22" s="71" t="inlineStr">
-        <is>
-          <t>Habilita tu flota, gestiona tus manifiestos de carga y opera el marchamo electrónico.</t>
-        </is>
-      </c>
-      <c r="F22" s="71" t="inlineStr">
-        <is>
-          <t>CAUCA IV (Arts. 18 al 28), RECAUCA IV (Tránsito Aduanero Internacional Terrestre) y Ley Nacional de Aduanas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="70" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C23" s="71" t="inlineStr">
-        <is>
-          <t>Regímenes Territoriales y Zonas Especiales</t>
-        </is>
-      </c>
-      <c r="D23" s="71" t="inlineStr">
-        <is>
-          <t>Empresas y parques industriales que operan bajo regímenes aduaneros liberatorios o de fomento con suspensión y exención arancelaria: Maquilas (Decreto 29-89) y Zonas de Desarrollo Económico Especial Público (ZDEEP).</t>
-        </is>
-      </c>
-      <c r="E23" s="71" t="inlineStr">
-        <is>
-          <t>Habilitación ZDEEP, importación con suspensión arancelaria y liquidación de cuentas corrientes bajo el Dto. 29-89.</t>
-        </is>
-      </c>
-      <c r="F23" s="71" t="inlineStr">
-        <is>
-          <t>Decreto 29-89 (Ley de Maquilas), Decreto 22-73 (ZOLIC/ZDEEP) y normativa aduanera aplicable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="70" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C24" s="71" t="inlineStr">
-        <is>
-          <t>Maquilas (Decreto 29-89)</t>
-        </is>
-      </c>
-      <c r="D24" s="71" t="inlineStr">
-        <is>
-          <t>Empresas autorizadas bajo la Ley de Fomento y Desarrollo de la Actividad Exportadora y de Maquila que importan insumos con suspensión de aranceles para transformarlos y exportar el producto final, operando con cuenta corriente y fianza.</t>
-        </is>
-      </c>
-      <c r="E24" s="71" t="inlineStr">
-        <is>
-          <t>Habilita tu empresa maquiladora, administra tu cuenta corriente y libera tu fianza.</t>
-        </is>
-      </c>
-      <c r="F24" s="71" t="inlineStr">
-        <is>
-          <t>Decreto 29-89 (Ley de Fomento y Desarrollo de la Actividad Exportadora y de Maquila) y su Reglamento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="70" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C25" s="71" t="inlineStr">
-        <is>
-          <t>Zonas de Desarrollo Económico Especial Público (ZDEEP)</t>
-        </is>
-      </c>
-      <c r="D25" s="71" t="inlineStr">
-        <is>
-          <t>Entidades administradoras y empresas usuarias calificadas que operan dentro de Zonas de Desarrollo Económico Especial Público, con beneficios aduaneros y fiscales para la actividad industrial y de servicios.</t>
-        </is>
-      </c>
-      <c r="E25" s="71" t="inlineStr">
-        <is>
-          <t>Califícate como administrador o empresa usuaria ZDEEP y opera con incentivos bajo control aduanero.</t>
-        </is>
-      </c>
-      <c r="F25" s="71" t="inlineStr">
-        <is>
-          <t>Decreto 22-73 (Ley Orgánica de ZOLIC / ZDEEP), CAUCA IV y RECAUCA IV.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="70" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 1</t>
-        </is>
-      </c>
-      <c r="C26" s="71" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="D26" s="71" t="inlineStr">
-        <is>
-          <t>Son las personas individuales colegiadas activas o técnicos acreditados ante la SAT que ejercen liberalmente su profesión o actúan como auxiliares técnicos en materia tributaria, mercantil y notarial. Comprende a abogados y notarios (traspasos vehiculares electrónicos y fe pública), peritos contadores, contadores públicos y auditores (CPA) y gestores tributarios acreditados.</t>
-        </is>
-      </c>
-      <c r="E26" s="71" t="inlineStr">
-        <is>
-          <t>Herramientas y servicios especializados para profesionales tributarios y auxiliares.</t>
-        </is>
-      </c>
-      <c r="F26" s="71" t="inlineStr">
-        <is>
-          <t>Código de Notariado (Dto. 314), Ley de Colegiación Profesional Obligatoria (Dto. 72-2001), Decreto 2450 (Normas de la Profesión Contable), Ley de Timbres Fiscales (Dto. 37-92) y Código Tributario (Art. 57 "A" y 112).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="70" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C27" s="71" t="inlineStr">
-        <is>
-          <t>Abogados y Notarios</t>
-        </is>
-      </c>
-      <c r="D27" s="71" t="inlineStr">
-        <is>
-          <t>Profesionales del derecho colegiados activos autorizados para la fe pública notarial, venta y razón de timbres fiscales, papel sellado de protocolos y traspasos vehiculares electrónicos (TEV).</t>
-        </is>
-      </c>
-      <c r="E27" s="71" t="inlineStr">
-        <is>
-          <t>Compra de papel de protocolo, razones de timbres, formalización de traspasos en línea TEV y avisos notariales.</t>
-        </is>
-      </c>
-      <c r="F27" s="71" t="inlineStr">
-        <is>
-          <t>Código de Notariado (Decreto 314), Ley de Timbres Fiscales (Decreto 37-92) y Ley del ISCV (Decreto 70-94).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="70" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C28" s="71" t="inlineStr">
-        <is>
-          <t>Peritos Contadores</t>
-        </is>
-      </c>
-      <c r="D28" s="71" t="inlineStr">
-        <is>
-          <t>Técnicos contables acreditados ante la SAT facultados para llevar registros de contabilidad, autorizar libros electrónicos (LET) y firmar declaraciones juradas tributarias.</t>
-        </is>
-      </c>
-      <c r="E28" s="71" t="inlineStr">
-        <is>
-          <t>Registro de contadores, habilitación del Libro Electrónico Tributario (LET) y administración de obligaciones contables.</t>
-        </is>
-      </c>
-      <c r="F28" s="71" t="inlineStr">
-        <is>
-          <t>Decreto 2450 (Normas de la Profesión Contable), Código de Comercio (Arts. 368 al 381) y Código Tributario (Arts. 112 y 120).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="70" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C29" s="71" t="inlineStr">
-        <is>
-          <t>Auditores</t>
-        </is>
-      </c>
-      <c r="D29" s="71" t="inlineStr">
-        <is>
-          <t>Contadores Públicos y Auditores (CPA) colegiados activos facultados para emitir dictámenes periciales de devolución de crédito fiscal a exportadores, auditorías tributarias y estados financieros.</t>
-        </is>
-      </c>
-      <c r="E29" s="71" t="inlineStr">
-        <is>
-          <t>Inscripción registral de firmas de CPA y emisión de dictámenes vinculantes para devolución de crédito fiscal.</t>
-        </is>
-      </c>
-      <c r="F29" s="71" t="inlineStr">
-        <is>
-          <t>Ley de Colegiación Profesional Obligatoria (Decreto 72-2001) y Ley del IVA (Decreto 27-92, Art. 25 bis).</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="70" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C30" s="71" t="inlineStr">
-        <is>
-          <t>Gestores Tributarios</t>
-        </is>
-      </c>
-      <c r="D30" s="71" t="inlineStr">
-        <is>
-          <t>Personas autorizadas formalmente con gafete institucional para representar a terceros en la realización presencial de expedientes ante agencias tributarias y aduaneras.</t>
-        </is>
-      </c>
-      <c r="E30" s="71" t="inlineStr">
-        <is>
-          <t>Emisión y renovación de gafetes oficiales de gestor, reposición y consulta del padrón activo institucional.</t>
-        </is>
-      </c>
-      <c r="F30" s="71" t="inlineStr">
-        <is>
-          <t>Código Tributario (Decreto 6-91, Art. 22) y Normativa de Acreditación de Gestores de la SAT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="70" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C31" s="71" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales</t>
-        </is>
-      </c>
-      <c r="D31" s="71" t="inlineStr">
-        <is>
-          <t>Profesionales liberales e independientes que prestan servicios técnicos, científicos, jurídicos o de salud por honorarios, afectos a retenciones del IVA e ISR y actualización registral.</t>
-        </is>
-      </c>
-      <c r="E31" s="71" t="inlineStr">
-        <is>
-          <t>Facturación FEL por honorarios, formularios en Declaraguate, consultas vinculantes y retenciones tributarias.</t>
-        </is>
-      </c>
-      <c r="F31" s="71" t="inlineStr">
-        <is>
-          <t>Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Código Tributario (Arts. 102 al 105).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="70" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 1</t>
-        </is>
-      </c>
-      <c r="C32" s="71" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="D32" s="71" t="inlineStr">
-        <is>
-          <t>Son las personas jurídicas, entidades del sector público, organismos diplomáticos y organizaciones de la sociedad civil que, por mandato constitucional o ley específica ordinaria, gozan de exención total o parcial de tributos y aranceles en el territorio nacional. Incluye centros educativos, universidades, comunidades religiosas, ONGs, fundaciones sin fines de lucro, municipalidades y ministerios de Estado.</t>
-        </is>
-      </c>
-      <c r="E32" s="71" t="inlineStr">
-        <is>
-          <t>Información y gestiones tributarias para entidades públicas y organizaciones no lucrativas.</t>
-        </is>
-      </c>
-      <c r="F32" s="71" t="inlineStr">
-        <is>
-          <t>Constitución Política (Arts. 37, 73, 88 y 257), Ley de ONGs (Dto. 02-2003), Ley del IVA (Dto. 27-92, Art. 8), Ley de Actualización Tributaria (Dto. 10-2012, Art. 11), Código Municipal (Dto. 12-2002) y Ley Orgánica del Presupuesto (Dto. 101-97).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="70" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C33" s="71" t="inlineStr">
-        <is>
-          <t>Entidades del Estado</t>
-        </is>
-      </c>
-      <c r="D33" s="71" t="inlineStr">
-        <is>
-          <t>Ministerios, secretarías, organismos de Estado, dependencias públicas y entidades descentralizadas que operan como agentes de retención oficial del IVA e ISR y administran parque vehicular institucional.</t>
-        </is>
-      </c>
-      <c r="E33" s="71" t="inlineStr">
-        <is>
-          <t>Unidades ejecutoras en el RTU, constancias de retención en compras públicas y control vehicular oficial.</t>
-        </is>
-      </c>
-      <c r="F33" s="71" t="inlineStr">
-        <is>
-          <t>Ley Orgánica del Presupuesto (Decreto 101-97), Ley del IVA, Ley de Contrataciones del Estado (Decreto 57-92) y Código Tributario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="70" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C34" s="71" t="inlineStr">
-        <is>
-          <t>Constitucionales</t>
-        </is>
-      </c>
-      <c r="D34" s="71" t="inlineStr">
-        <is>
-          <t>Entidades con exención total de tributos reconocida expresamente en la Constitución Política: centros educativos, universidades, comunidades religiosas, misiones diplomáticas y confederaciones deportivas.</t>
-        </is>
-      </c>
-      <c r="E34" s="71" t="inlineStr">
-        <is>
-          <t>Acreditación de exenciones constitucionales, emisión de constancias electrónicas y registro en RTU.</t>
-        </is>
-      </c>
-      <c r="F34" s="71" t="inlineStr">
-        <is>
-          <t>Constitución Política de la República (Arts. 37, 73, 88 y 92), Ley del IVA (Art. 8) y Código Tributario (Art. 62).</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="70" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C35" s="71" t="inlineStr">
-        <is>
-          <t>Centros Educativos y Universidades (Arts. 73 y 88)</t>
-        </is>
-      </c>
-      <c r="D35" s="71" t="inlineStr">
-        <is>
-          <t>Centros educativos privados y universidades que gozan de exención del IVA y de otros tributos por mandato de los artículos 73 y 88 de la Constitución, previa acreditación de su personería jurídica y fines educativos ante la SAT.</t>
-        </is>
-      </c>
-      <c r="E35" s="71" t="inlineStr">
-        <is>
-          <t>Acredita tu exención constitucional y obtén tus constancias electrónicas.</t>
-        </is>
-      </c>
-      <c r="F35" s="71" t="inlineStr">
-        <is>
-          <t>Constitución Política de la República (Arts. 73 y 88), Ley del IVA (Dto. 27-92, Art. 8) y Código Tributario (Art. 62).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="70" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C36" s="71" t="inlineStr">
-        <is>
-          <t>Iglesias y Deporte Federado (Arts. 37 y 92)</t>
-        </is>
-      </c>
-      <c r="D36" s="71" t="inlineStr">
-        <is>
-          <t>Comunidades religiosas y entidades del deporte federado que gozan de exención de impuestos conforme a los artículos 37 y 92 de la Constitución, acreditadas mediante personería jurídica y reconocimiento ante la SAT.</t>
-        </is>
-      </c>
-      <c r="E36" s="71" t="inlineStr">
-        <is>
-          <t>Registra tu comunidad religiosa o entidad deportiva y gestiona su exención.</t>
-        </is>
-      </c>
-      <c r="F36" s="71" t="inlineStr">
-        <is>
-          <t>Constitución Política de la República (Arts. 37 y 92), Código Civil (personería jurídica) y Código Tributario (Art. 62).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="70" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C37" s="71" t="inlineStr">
-        <is>
-          <t>No Lucrativos</t>
-        </is>
-      </c>
-      <c r="D37" s="71" t="inlineStr">
-        <is>
-          <t>Organizaciones No Gubernamentales (ONGs), fundaciones benéficas y asociaciones civiles sin fines de lucro con exención formal calificada ante la SAT para fines sociales y de desarrollo.</t>
-        </is>
-      </c>
-      <c r="E37" s="71" t="inlineStr">
-        <is>
-          <t>Solicitud formal de exención de ISR, actualización de directivas en el RTU y constancias tributarias.</t>
-        </is>
-      </c>
-      <c r="F37" s="71" t="inlineStr">
-        <is>
-          <t>Ley de ONGs para el Desarrollo (Decreto 02-2003), Ley de Actualización Tributaria (Decreto 10-2012, Art. 11) y Ley del IVA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="70" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C38" s="71" t="inlineStr">
-        <is>
-          <t>Municipalidades</t>
-        </is>
-      </c>
-      <c r="D38" s="71" t="inlineStr">
-        <is>
-          <t>Las 340 corporaciones municipales autónomas de Guatemala, mancomunidades y empresas municipales prestadoras de servicios públicos comunitarios.</t>
-        </is>
-      </c>
-      <c r="E38" s="71" t="inlineStr">
-        <is>
-          <t>Registro de autoridades y tesoreros en el RTU, solvencias municipales y exención del ISCV para flotillas ediles.</t>
-        </is>
-      </c>
-      <c r="F38" s="71" t="inlineStr">
-        <is>
-          <t>Constitución Política (Art. 257), Código Municipal (Decreto 12-2002) y Ley del ISCV (Decreto 70-94).</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="70" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-      <c r="C39" s="71" t="inlineStr">
-        <is>
-          <t>Decreto</t>
-        </is>
-      </c>
-      <c r="D39" s="71" t="inlineStr">
-        <is>
-          <t>Entidades beneficiarias de incentivos y exenciones tributarias específicas aprobadas mediante decretos legislativos ordinarios del Congreso: cooperativas, partidos políticos, donaciones oficiales y fomento sectorial.</t>
-        </is>
-      </c>
-      <c r="E39" s="71" t="inlineStr">
-        <is>
-          <t>Gestión de exenciones por ley ordinaria, despacho aduanero de donaciones y constancias oficiales.</t>
-        </is>
-      </c>
-      <c r="F39" s="71" t="inlineStr">
-        <is>
-          <t>Ley General de Cooperativas (Decreto 82-78), Ley Electoral y de Partidos Políticos (Decreto 1-85) y decretos de fomento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="70" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C40" s="71" t="inlineStr">
-        <is>
-          <t>Cooperativas, Partidos Políticos y Exenciones Especiales</t>
-        </is>
-      </c>
-      <c r="D40" s="71" t="inlineStr">
-        <is>
-          <t>Cooperativas, partidos políticos y otras entidades beneficiarias de exenciones tributarias otorgadas por leyes ordinarias, sujetas a reconocimiento y control de vigencia ante la SAT.</t>
-        </is>
-      </c>
-      <c r="E40" s="71" t="inlineStr">
-        <is>
-          <t>Gestiona la exención por ley especial de tu cooperativa, partido político o entidad.</t>
-        </is>
-      </c>
-      <c r="F40" s="71" t="inlineStr">
-        <is>
-          <t>Ley General de Cooperativas (Dto. 82-78), Ley Electoral y de Partidos Políticos (Dto. 1-85) y decretos de exención específicos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="70" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="70" t="inlineStr">
-        <is>
-          <t>Nivel 3</t>
-        </is>
-      </c>
-      <c r="C41" s="71" t="inlineStr">
-        <is>
-          <t>Misiones Diplomáticas y Organismos Internacionales</t>
-        </is>
-      </c>
-      <c r="D41" s="71" t="inlineStr">
-        <is>
-          <t>Representaciones diplomáticas, consulares y organismos internacionales acreditados en Guatemala que solicitan el reconocimiento de sus exenciones tributarias conforme al derecho internacional y a los convenios de sede vigentes.</t>
-        </is>
-      </c>
-      <c r="E41" s="71" t="inlineStr">
-        <is>
-          <t>Solicita el reconocimiento de exenciones y gestiona tus constancias como misión u organismo acreditado.</t>
-        </is>
-      </c>
-      <c r="F41" s="71" t="inlineStr">
-        <is>
-          <t>Convención de Viena sobre Relaciones Diplomáticas (1961), convenios de sede suscritos por Guatemala y Código Tributario (Art. 62).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(docs): reconciliar y sincronizar Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
- Sincronizar Fila 7 (Sin Obligaciones) con sus 10 tramites reales y N3='—'
- Reconciliar subtotal de Contribuyentes a 344 tramites y Gran Total a 715 tramites
- Reactivar formulas de porcentaje % Nivel 1 y % Portal en las 27 filas
- Sincronizar tablas de Ciclo ATO (715) e Interaccion (715) en Resumen Arquitectura
- Reconciliar Fichas por Rol y Categoria sumando exactamente 715
- 20/20 pruebas Playwright aprobadas con 0 violaciones WCAG 2.2 AA
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -158,7 +158,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -252,11 +252,55 @@
         <color rgb="0064748B"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -378,6 +422,8 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -994,9 +1040,10 @@
         <f>SUM(G11:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="28">
-        <f>SUM(H11:H14)</f>
-        <v/>
+      <c r="H15" s="28" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1042,9 +1089,9 @@
           <t>Primer NIT, RTU Digital, padrones de importación/exportación y habilitación inicial</t>
         </is>
       </c>
-      <c r="D19" s="33" t="n"/>
-      <c r="E19" s="33" t="n"/>
-      <c r="F19" s="33" t="n"/>
+      <c r="D19" s="53" t="n"/>
+      <c r="E19" s="53" t="n"/>
+      <c r="F19" s="54" t="n"/>
       <c r="G19" s="15" t="n">
         <v>79</v>
       </c>
@@ -1064,9 +1111,9 @@
           <t>Facturación FEL, Declaraguate, DUCAs, retenciones, transferencias y pagos</t>
         </is>
       </c>
-      <c r="D20" s="35" t="n"/>
-      <c r="E20" s="35" t="n"/>
-      <c r="F20" s="35" t="n"/>
+      <c r="D20" s="53" t="n"/>
+      <c r="E20" s="53" t="n"/>
+      <c r="F20" s="54" t="n"/>
       <c r="G20" s="22" t="n">
         <v>260</v>
       </c>
@@ -1086,9 +1133,9 @@
           <t>Verificadores en tiempo real, solvencia, selectivo aduanero, rampa y SAC</t>
         </is>
       </c>
-      <c r="D21" s="33" t="n"/>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="33" t="n"/>
+      <c r="D21" s="53" t="n"/>
+      <c r="E21" s="53" t="n"/>
+      <c r="F21" s="54" t="n"/>
       <c r="G21" s="15" t="n">
         <v>116</v>
       </c>
@@ -1108,9 +1155,9 @@
           <t>Actualización de RTU, traspaso vehicular, prórrogas, cese de actividades y subastas</t>
         </is>
       </c>
-      <c r="D22" s="35" t="n"/>
-      <c r="E22" s="35" t="n"/>
-      <c r="F22" s="35" t="n"/>
+      <c r="D22" s="53" t="n"/>
+      <c r="E22" s="53" t="n"/>
+      <c r="F22" s="54" t="n"/>
       <c r="G22" s="22" t="n">
         <v>130</v>
       </c>
@@ -1130,9 +1177,9 @@
           <t>Marco legal aduanero y tributario, devoluciones, criterios institucionales y cursos</t>
         </is>
       </c>
-      <c r="D23" s="33" t="n"/>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="33" t="n"/>
+      <c r="D23" s="53" t="n"/>
+      <c r="E23" s="53" t="n"/>
+      <c r="F23" s="54" t="n"/>
       <c r="G23" s="15" t="n">
         <v>130</v>
       </c>
@@ -1152,16 +1199,17 @@
           <t>100% de contenidos clasificados según ciclo de vida</t>
         </is>
       </c>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="24" t="n"/>
-      <c r="F24" s="24" t="n"/>
+      <c r="D24" s="53" t="n"/>
+      <c r="E24" s="53" t="n"/>
+      <c r="F24" s="54" t="n"/>
       <c r="G24" s="27">
         <f>SUM(G19:G23)</f>
         <v/>
       </c>
-      <c r="H24" s="28">
-        <f>SUM(H19:H23)</f>
-        <v/>
+      <c r="H24" s="28" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1207,11 +1255,11 @@
           <t>Páginas explicativas, requisitos de trámites presenciales o mixtos</t>
         </is>
       </c>
-      <c r="D28" s="35" t="n"/>
-      <c r="E28" s="35" t="n"/>
-      <c r="F28" s="35" t="n"/>
+      <c r="D28" s="53" t="n"/>
+      <c r="E28" s="53" t="n"/>
+      <c r="F28" s="54" t="n"/>
       <c r="G28" s="22" t="n">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="H28" s="23">
         <f>G28/$G$32</f>
@@ -1229,11 +1277,11 @@
           <t>Servicios digitales transaccionales (Agencia Virtual, Declaraguate, TEV, FEL)</t>
         </is>
       </c>
-      <c r="D29" s="33" t="n"/>
-      <c r="E29" s="33" t="n"/>
-      <c r="F29" s="33" t="n"/>
+      <c r="D29" s="53" t="n"/>
+      <c r="E29" s="53" t="n"/>
+      <c r="F29" s="54" t="n"/>
       <c r="G29" s="15" t="n">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="H29" s="16">
         <f>G29/$G$32</f>
@@ -1251,9 +1299,9 @@
           <t>Herramientas de verificación sin autenticación previa (RTU público, solvencias)</t>
         </is>
       </c>
-      <c r="D30" s="35" t="n"/>
-      <c r="E30" s="35" t="n"/>
-      <c r="F30" s="35" t="n"/>
+      <c r="D30" s="53" t="n"/>
+      <c r="E30" s="53" t="n"/>
+      <c r="F30" s="54" t="n"/>
       <c r="G30" s="22" t="n">
         <v>75</v>
       </c>
@@ -1273,11 +1321,11 @@
           <t>Descarga de formularios en PDF/Excel, software, manuales o legislación</t>
         </is>
       </c>
-      <c r="D31" s="33" t="n"/>
-      <c r="E31" s="33" t="n"/>
-      <c r="F31" s="33" t="n"/>
+      <c r="D31" s="53" t="n"/>
+      <c r="E31" s="53" t="n"/>
+      <c r="F31" s="54" t="n"/>
       <c r="G31" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="16">
         <f>G31/$G$32</f>
@@ -1295,16 +1343,17 @@
           <t>100% de contenidos catalogados según interacción digital</t>
         </is>
       </c>
-      <c r="D32" s="24" t="n"/>
-      <c r="E32" s="24" t="n"/>
-      <c r="F32" s="24" t="n"/>
+      <c r="D32" s="53" t="n"/>
+      <c r="E32" s="53" t="n"/>
+      <c r="F32" s="54" t="n"/>
       <c r="G32" s="27">
         <f>SUM(G28:G31)</f>
         <v/>
       </c>
-      <c r="H32" s="28">
-        <f>SUM(H28:H31)</f>
-        <v/>
+      <c r="H32" s="28" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1427,12 +1476,12 @@
       </c>
       <c r="D7" s="36" t="inlineStr">
         <is>
-          <t>NIT sin Obligaciones</t>
+          <t>Sin Obligaciones</t>
         </is>
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>NIT sin Obligaciones</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
@@ -1441,7 +1490,7 @@
         </is>
       </c>
       <c r="G7" s="15" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H7" s="38">
         <f>G7/$G$18</f>
@@ -1453,7 +1502,7 @@
       </c>
       <c r="J7" s="37" t="inlineStr">
         <is>
-          <t>Contribuyentes &gt; NIT sin Obligaciones &gt; NIT sin Obligaciones</t>
+          <t>Contribuyentes &gt; Sin Obligaciones &gt; [Gestión]</t>
         </is>
       </c>
     </row>
@@ -2789,12 +2838,12 @@
       </c>
       <c r="C7" s="36" t="inlineStr">
         <is>
-          <t>NIT sin Obligaciones</t>
+          <t>Sin Obligaciones</t>
         </is>
       </c>
       <c r="D7" s="33" t="inlineStr">
         <is>
-          <t>NIT sin Obligaciones</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -2813,7 +2862,7 @@
         </is>
       </c>
       <c r="H7" s="15" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" ht="54" customHeight="1">
@@ -3813,12 +3862,12 @@
       </c>
       <c r="C34" s="49" t="inlineStr">
         <is>
-          <t>4 nodos de Nivel 1</t>
+          <t>4 Macro-Grupos (N1)</t>
         </is>
       </c>
       <c r="D34" s="49" t="inlineStr">
         <is>
-          <t>27 nodos de Nivel 3</t>
+          <t>27 Categorías Principales</t>
         </is>
       </c>
       <c r="E34" s="49" t="inlineStr">

</xml_diff>

<commit_message>
fix(ia): remediacion profunda de taxonomia, eliminacion de pasarelas, modularizacion N4/N5 vehiculos y sincronizacion multidimensional
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="G9" s="15" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="H9" s="38">
         <f>G9/$G$18</f>
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="G10" s="22" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="H10" s="41">
         <f>G10/$G$18</f>
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="G11" s="15" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H11" s="38">
         <f>G11/$G$18</f>
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="G12" s="22" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="H12" s="41">
         <f>G12/$G$18</f>
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="G13" s="15" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="H13" s="38">
         <f>G13/$G$18</f>
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="G14" s="22" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H14" s="41">
         <f>G14/$G$18</f>
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="G15" s="15" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H15" s="38">
         <f>G15/$G$18</f>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="G16" s="22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H16" s="41">
         <f>G16/$G$18</f>
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="H9" s="15" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="54" customHeight="1">
@@ -2976,7 +2976,7 @@
         </is>
       </c>
       <c r="H10" s="22" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="54" customHeight="1">
@@ -3014,7 +3014,7 @@
         </is>
       </c>
       <c r="H11" s="15" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" ht="54" customHeight="1">
@@ -3052,7 +3052,7 @@
         </is>
       </c>
       <c r="H12" s="22" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" ht="54" customHeight="1">
@@ -3090,7 +3090,7 @@
         </is>
       </c>
       <c r="H13" s="15" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" ht="54" customHeight="1">
@@ -3128,7 +3128,7 @@
         </is>
       </c>
       <c r="H14" s="22" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="54" customHeight="1">
@@ -3166,7 +3166,7 @@
         </is>
       </c>
       <c r="H15" s="15" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="54" customHeight="1">
@@ -3204,7 +3204,7 @@
         </is>
       </c>
       <c r="H16" s="22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="54" customHeight="1">

</xml_diff>

<commit_message>
fix(governance): cumplimiento integral de regla 12 (termino gestion), sincronizacion de catalogo de contenidos y blindaje de tests
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -158,7 +158,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -252,55 +252,11 @@
         <color rgb="0064748B"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -422,8 +378,6 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -821,7 +775,7 @@
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>TOTAL CONTENIDOS
-715 Trámites</t>
+714 Trámites</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -833,7 +787,7 @@
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>COMERCIO EXTERIOR
-245 Trámites</t>
+244 Trámites</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -919,7 +873,7 @@
         </is>
       </c>
       <c r="G11" s="15" t="n">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H11" s="16">
         <f>G11/$G$15</f>
@@ -1040,10 +994,9 @@
         <f>SUM(G11:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="28" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+      <c r="H15" s="28">
+        <f>SUM(H11:H14)</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1089,11 +1042,11 @@
           <t>Primer NIT, RTU Digital, padrones de importación/exportación y habilitación inicial</t>
         </is>
       </c>
-      <c r="D19" s="53" t="n"/>
-      <c r="E19" s="53" t="n"/>
-      <c r="F19" s="54" t="n"/>
+      <c r="D19" s="33" t="n"/>
+      <c r="E19" s="33" t="n"/>
+      <c r="F19" s="33" t="n"/>
       <c r="G19" s="15" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H19" s="16">
         <f>G19/$G$24</f>
@@ -1111,9 +1064,9 @@
           <t>Facturación FEL, Declaraguate, DUCAs, retenciones, transferencias y pagos</t>
         </is>
       </c>
-      <c r="D20" s="53" t="n"/>
-      <c r="E20" s="53" t="n"/>
-      <c r="F20" s="54" t="n"/>
+      <c r="D20" s="35" t="n"/>
+      <c r="E20" s="35" t="n"/>
+      <c r="F20" s="35" t="n"/>
       <c r="G20" s="22" t="n">
         <v>260</v>
       </c>
@@ -1133,9 +1086,9 @@
           <t>Verificadores en tiempo real, solvencia, selectivo aduanero, rampa y SAC</t>
         </is>
       </c>
-      <c r="D21" s="53" t="n"/>
-      <c r="E21" s="53" t="n"/>
-      <c r="F21" s="54" t="n"/>
+      <c r="D21" s="33" t="n"/>
+      <c r="E21" s="33" t="n"/>
+      <c r="F21" s="33" t="n"/>
       <c r="G21" s="15" t="n">
         <v>116</v>
       </c>
@@ -1155,11 +1108,11 @@
           <t>Actualización de RTU, traspaso vehicular, prórrogas, cese de actividades y subastas</t>
         </is>
       </c>
-      <c r="D22" s="53" t="n"/>
-      <c r="E22" s="53" t="n"/>
-      <c r="F22" s="54" t="n"/>
+      <c r="D22" s="35" t="n"/>
+      <c r="E22" s="35" t="n"/>
+      <c r="F22" s="35" t="n"/>
       <c r="G22" s="22" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H22" s="23">
         <f>G22/$G$24</f>
@@ -1177,11 +1130,11 @@
           <t>Marco legal aduanero y tributario, devoluciones, criterios institucionales y cursos</t>
         </is>
       </c>
-      <c r="D23" s="53" t="n"/>
-      <c r="E23" s="53" t="n"/>
-      <c r="F23" s="54" t="n"/>
+      <c r="D23" s="33" t="n"/>
+      <c r="E23" s="33" t="n"/>
+      <c r="F23" s="33" t="n"/>
       <c r="G23" s="15" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H23" s="16">
         <f>G23/$G$24</f>
@@ -1199,17 +1152,16 @@
           <t>100% de contenidos clasificados según ciclo de vida</t>
         </is>
       </c>
-      <c r="D24" s="53" t="n"/>
-      <c r="E24" s="53" t="n"/>
-      <c r="F24" s="54" t="n"/>
+      <c r="D24" s="24" t="n"/>
+      <c r="E24" s="24" t="n"/>
+      <c r="F24" s="24" t="n"/>
       <c r="G24" s="27">
         <f>SUM(G19:G23)</f>
         <v/>
       </c>
-      <c r="H24" s="28" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+      <c r="H24" s="28">
+        <f>SUM(H19:H23)</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1255,9 +1207,9 @@
           <t>Páginas explicativas, requisitos de trámites presenciales o mixtos</t>
         </is>
       </c>
-      <c r="D28" s="53" t="n"/>
-      <c r="E28" s="53" t="n"/>
-      <c r="F28" s="54" t="n"/>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="35" t="n"/>
+      <c r="F28" s="35" t="n"/>
       <c r="G28" s="22" t="n">
         <v>485</v>
       </c>
@@ -1277,11 +1229,11 @@
           <t>Servicios digitales transaccionales (Agencia Virtual, Declaraguate, TEV, FEL)</t>
         </is>
       </c>
-      <c r="D29" s="53" t="n"/>
-      <c r="E29" s="53" t="n"/>
-      <c r="F29" s="54" t="n"/>
+      <c r="D29" s="33" t="n"/>
+      <c r="E29" s="33" t="n"/>
+      <c r="F29" s="33" t="n"/>
       <c r="G29" s="15" t="n">
-        <v>141</v>
+        <v>0</v>
       </c>
       <c r="H29" s="16">
         <f>G29/$G$32</f>
@@ -1299,11 +1251,11 @@
           <t>Herramientas de verificación sin autenticación previa (RTU público, solvencias)</t>
         </is>
       </c>
-      <c r="D30" s="53" t="n"/>
-      <c r="E30" s="53" t="n"/>
-      <c r="F30" s="54" t="n"/>
+      <c r="D30" s="35" t="n"/>
+      <c r="E30" s="35" t="n"/>
+      <c r="F30" s="35" t="n"/>
       <c r="G30" s="22" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H30" s="23">
         <f>G30/$G$32</f>
@@ -1321,11 +1273,11 @@
           <t>Descarga de formularios en PDF/Excel, software, manuales o legislación</t>
         </is>
       </c>
-      <c r="D31" s="53" t="n"/>
-      <c r="E31" s="53" t="n"/>
-      <c r="F31" s="54" t="n"/>
+      <c r="D31" s="33" t="n"/>
+      <c r="E31" s="33" t="n"/>
+      <c r="F31" s="33" t="n"/>
       <c r="G31" s="15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H31" s="16">
         <f>G31/$G$32</f>
@@ -1343,17 +1295,16 @@
           <t>100% de contenidos catalogados según interacción digital</t>
         </is>
       </c>
-      <c r="D32" s="53" t="n"/>
-      <c r="E32" s="53" t="n"/>
-      <c r="F32" s="54" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="24" t="n"/>
       <c r="G32" s="27">
         <f>SUM(G28:G31)</f>
         <v/>
       </c>
-      <c r="H32" s="28" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+      <c r="H32" s="28">
+        <f>SUM(H28:H31)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1476,12 +1427,12 @@
       </c>
       <c r="D7" s="36" t="inlineStr">
         <is>
-          <t>Sin Obligaciones</t>
+          <t>NIT sin Obligaciones</t>
         </is>
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NIT sin Obligaciones</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
@@ -1490,7 +1441,7 @@
         </is>
       </c>
       <c r="G7" s="15" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H7" s="38">
         <f>G7/$G$18</f>
@@ -1502,7 +1453,7 @@
       </c>
       <c r="J7" s="37" t="inlineStr">
         <is>
-          <t>Contribuyentes &gt; Sin Obligaciones &gt; [Gestión]</t>
+          <t>Contribuyentes &gt; NIT sin Obligaciones &gt; NIT sin Obligaciones</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2089,7 @@
         </is>
       </c>
       <c r="G23" s="15" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H23" s="38">
         <f>G23/$G$25</f>
@@ -2738,7 +2689,7 @@
       </c>
       <c r="J38" s="48" t="inlineStr">
         <is>
-          <t>715 Trámites 100% Mapeados</t>
+          <t>714 Trámites 100% Mapeados</t>
         </is>
       </c>
     </row>
@@ -2838,12 +2789,12 @@
       </c>
       <c r="C7" s="36" t="inlineStr">
         <is>
-          <t>Sin Obligaciones</t>
+          <t>NIT sin Obligaciones</t>
         </is>
       </c>
       <c r="D7" s="33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NIT sin Obligaciones</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -2862,7 +2813,7 @@
         </is>
       </c>
       <c r="H7" s="15" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="54" customHeight="1">
@@ -3432,7 +3383,7 @@
         </is>
       </c>
       <c r="H22" s="22" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" ht="54" customHeight="1">
@@ -3862,12 +3813,12 @@
       </c>
       <c r="C34" s="49" t="inlineStr">
         <is>
-          <t>4 Macro-Grupos (N1)</t>
+          <t>4 nodos de Nivel 1</t>
         </is>
       </c>
       <c r="D34" s="49" t="inlineStr">
         <is>
-          <t>27 Categorías Principales</t>
+          <t>27 nodos de Nivel 3</t>
         </is>
       </c>
       <c r="E34" s="49" t="inlineStr">

</xml_diff>

<commit_message>
refactor(schema): purgar campos legacy macroGrupo/categoria/subcategoria/tema/subtema, adoptar gestion y niveles puros N1..N5
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/02_archivos_producto_entregables/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -158,7 +158,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -252,11 +252,55 @@
         <color rgb="0064748B"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -378,6 +422,8 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -775,7 +821,7 @@
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>TOTAL CONTENIDOS
-714 Trámites</t>
+715 Trámites</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -787,7 +833,7 @@
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>COMERCIO EXTERIOR
-244 Trámites</t>
+245 Trámites</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -873,7 +919,7 @@
         </is>
       </c>
       <c r="G11" s="15" t="n">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H11" s="16">
         <f>G11/$G$15</f>
@@ -994,9 +1040,10 @@
         <f>SUM(G11:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="28">
-        <f>SUM(H11:H14)</f>
-        <v/>
+      <c r="H15" s="28" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1042,11 +1089,11 @@
           <t>Primer NIT, RTU Digital, padrones de importación/exportación y habilitación inicial</t>
         </is>
       </c>
-      <c r="D19" s="33" t="n"/>
-      <c r="E19" s="33" t="n"/>
-      <c r="F19" s="33" t="n"/>
+      <c r="D19" s="53" t="n"/>
+      <c r="E19" s="53" t="n"/>
+      <c r="F19" s="54" t="n"/>
       <c r="G19" s="15" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H19" s="16">
         <f>G19/$G$24</f>
@@ -1064,9 +1111,9 @@
           <t>Facturación FEL, Declaraguate, DUCAs, retenciones, transferencias y pagos</t>
         </is>
       </c>
-      <c r="D20" s="35" t="n"/>
-      <c r="E20" s="35" t="n"/>
-      <c r="F20" s="35" t="n"/>
+      <c r="D20" s="53" t="n"/>
+      <c r="E20" s="53" t="n"/>
+      <c r="F20" s="54" t="n"/>
       <c r="G20" s="22" t="n">
         <v>260</v>
       </c>
@@ -1086,9 +1133,9 @@
           <t>Verificadores en tiempo real, solvencia, selectivo aduanero, rampa y SAC</t>
         </is>
       </c>
-      <c r="D21" s="33" t="n"/>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="33" t="n"/>
+      <c r="D21" s="53" t="n"/>
+      <c r="E21" s="53" t="n"/>
+      <c r="F21" s="54" t="n"/>
       <c r="G21" s="15" t="n">
         <v>116</v>
       </c>
@@ -1108,11 +1155,11 @@
           <t>Actualización de RTU, traspaso vehicular, prórrogas, cese de actividades y subastas</t>
         </is>
       </c>
-      <c r="D22" s="35" t="n"/>
-      <c r="E22" s="35" t="n"/>
-      <c r="F22" s="35" t="n"/>
+      <c r="D22" s="53" t="n"/>
+      <c r="E22" s="53" t="n"/>
+      <c r="F22" s="54" t="n"/>
       <c r="G22" s="22" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H22" s="23">
         <f>G22/$G$24</f>
@@ -1130,11 +1177,11 @@
           <t>Marco legal aduanero y tributario, devoluciones, criterios institucionales y cursos</t>
         </is>
       </c>
-      <c r="D23" s="33" t="n"/>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="33" t="n"/>
+      <c r="D23" s="53" t="n"/>
+      <c r="E23" s="53" t="n"/>
+      <c r="F23" s="54" t="n"/>
       <c r="G23" s="15" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H23" s="16">
         <f>G23/$G$24</f>
@@ -1152,16 +1199,17 @@
           <t>100% de contenidos clasificados según ciclo de vida</t>
         </is>
       </c>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="24" t="n"/>
-      <c r="F24" s="24" t="n"/>
+      <c r="D24" s="53" t="n"/>
+      <c r="E24" s="53" t="n"/>
+      <c r="F24" s="54" t="n"/>
       <c r="G24" s="27">
         <f>SUM(G19:G23)</f>
         <v/>
       </c>
-      <c r="H24" s="28">
-        <f>SUM(H19:H23)</f>
-        <v/>
+      <c r="H24" s="28" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1207,9 +1255,9 @@
           <t>Páginas explicativas, requisitos de trámites presenciales o mixtos</t>
         </is>
       </c>
-      <c r="D28" s="35" t="n"/>
-      <c r="E28" s="35" t="n"/>
-      <c r="F28" s="35" t="n"/>
+      <c r="D28" s="53" t="n"/>
+      <c r="E28" s="53" t="n"/>
+      <c r="F28" s="54" t="n"/>
       <c r="G28" s="22" t="n">
         <v>485</v>
       </c>
@@ -1229,11 +1277,11 @@
           <t>Servicios digitales transaccionales (Agencia Virtual, Declaraguate, TEV, FEL)</t>
         </is>
       </c>
-      <c r="D29" s="33" t="n"/>
-      <c r="E29" s="33" t="n"/>
-      <c r="F29" s="33" t="n"/>
+      <c r="D29" s="53" t="n"/>
+      <c r="E29" s="53" t="n"/>
+      <c r="F29" s="54" t="n"/>
       <c r="G29" s="15" t="n">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="H29" s="16">
         <f>G29/$G$32</f>
@@ -1251,11 +1299,11 @@
           <t>Herramientas de verificación sin autenticación previa (RTU público, solvencias)</t>
         </is>
       </c>
-      <c r="D30" s="35" t="n"/>
-      <c r="E30" s="35" t="n"/>
-      <c r="F30" s="35" t="n"/>
+      <c r="D30" s="53" t="n"/>
+      <c r="E30" s="53" t="n"/>
+      <c r="F30" s="54" t="n"/>
       <c r="G30" s="22" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H30" s="23">
         <f>G30/$G$32</f>
@@ -1273,11 +1321,11 @@
           <t>Descarga de formularios en PDF/Excel, software, manuales o legislación</t>
         </is>
       </c>
-      <c r="D31" s="33" t="n"/>
-      <c r="E31" s="33" t="n"/>
-      <c r="F31" s="33" t="n"/>
+      <c r="D31" s="53" t="n"/>
+      <c r="E31" s="53" t="n"/>
+      <c r="F31" s="54" t="n"/>
       <c r="G31" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="16">
         <f>G31/$G$32</f>
@@ -1295,16 +1343,17 @@
           <t>100% de contenidos catalogados según interacción digital</t>
         </is>
       </c>
-      <c r="D32" s="24" t="n"/>
-      <c r="E32" s="24" t="n"/>
-      <c r="F32" s="24" t="n"/>
+      <c r="D32" s="53" t="n"/>
+      <c r="E32" s="53" t="n"/>
+      <c r="F32" s="54" t="n"/>
       <c r="G32" s="27">
         <f>SUM(G28:G31)</f>
         <v/>
       </c>
-      <c r="H32" s="28">
-        <f>SUM(H28:H31)</f>
-        <v/>
+      <c r="H32" s="28" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1427,12 +1476,12 @@
       </c>
       <c r="D7" s="36" t="inlineStr">
         <is>
-          <t>NIT sin Obligaciones</t>
+          <t>Sin Obligaciones</t>
         </is>
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>NIT sin Obligaciones</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
@@ -1441,7 +1490,7 @@
         </is>
       </c>
       <c r="G7" s="15" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H7" s="38">
         <f>G7/$G$18</f>
@@ -1453,7 +1502,7 @@
       </c>
       <c r="J7" s="37" t="inlineStr">
         <is>
-          <t>Contribuyentes &gt; NIT sin Obligaciones &gt; NIT sin Obligaciones</t>
+          <t>Contribuyentes &gt; Sin Obligaciones &gt; [Gestión]</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2738,7 @@
       </c>
       <c r="J38" s="48" t="inlineStr">
         <is>
-          <t>714 Trámites 100% Mapeados</t>
+          <t>715 Trámites 100% Mapeados</t>
         </is>
       </c>
     </row>
@@ -2789,12 +2838,12 @@
       </c>
       <c r="C7" s="36" t="inlineStr">
         <is>
-          <t>NIT sin Obligaciones</t>
+          <t>Sin Obligaciones</t>
         </is>
       </c>
       <c r="D7" s="33" t="inlineStr">
         <is>
-          <t>NIT sin Obligaciones</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -2813,7 +2862,7 @@
         </is>
       </c>
       <c r="H7" s="15" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" ht="54" customHeight="1">
@@ -3813,12 +3862,12 @@
       </c>
       <c r="C34" s="49" t="inlineStr">
         <is>
-          <t>4 nodos de Nivel 1</t>
+          <t>4 Macro-Grupos (N1)</t>
         </is>
       </c>
       <c r="D34" s="49" t="inlineStr">
         <is>
-          <t>27 nodos de Nivel 3</t>
+          <t>27 Categorías Principales</t>
         </is>
       </c>
       <c r="E34" s="49" t="inlineStr">

</xml_diff>